<commit_message>
Use allocate available for H2 dispatch to allocate when surviving capacity > demand; update electrolyzer cost
</commit_message>
<xml_diff>
--- a/InputData/hydgn/HPEC/Hydrogen Production Eqpt Costs.xlsx
+++ b/InputData/hydgn/HPEC/Hydrogen Production Eqpt Costs.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\hydgn\HPEC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\hydgn\HPEC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A06FFE47-8401-4153-B365-3B8D108180A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C0CA885-5B69-4DE6-A0C9-AA7D40979DE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30315" yWindow="315" windowWidth="21630" windowHeight="13245" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="IEA Data" sheetId="2" r:id="rId2"/>
-    <sheet name="Conversion Factors" sheetId="4" r:id="rId3"/>
-    <sheet name="HPEC" sheetId="3" r:id="rId4"/>
-    <sheet name="HPEO" sheetId="5" r:id="rId5"/>
+    <sheet name="DoE Data" sheetId="6" r:id="rId3"/>
+    <sheet name="Conversion Factors" sheetId="4" r:id="rId4"/>
+    <sheet name="HPEC" sheetId="3" r:id="rId5"/>
+    <sheet name="HPEO" sheetId="5" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="btu_per_kwh">'Conversion Factors'!$A$3</definedName>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="86">
   <si>
     <t>HPEC Hydrogen Production Equipment CapEx</t>
   </si>
@@ -291,12 +292,48 @@
   <si>
     <t>have ~15% lower capital costs and ~5% lower production costs than SMRs.</t>
   </si>
+  <si>
+    <t>Department of Energy</t>
+  </si>
+  <si>
+    <t>Clean Hydrogen Production Cost PEM Electrolyzer</t>
+  </si>
+  <si>
+    <t>https://www.hydrogen.energy.gov/docs/hydrogenprogramlibraries/pdfs/24005-clean-hydrogen-production-cost-pem-electrolyzer.pdf</t>
+  </si>
+  <si>
+    <t>Table 2</t>
+  </si>
+  <si>
+    <t>For DoE data we convert from 2022 to 2012 dollars:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$/kW </t>
+  </si>
+  <si>
+    <t>2022 USD</t>
+  </si>
+  <si>
+    <t>2012 USD</t>
+  </si>
+  <si>
+    <t>2024 cost</t>
+  </si>
+  <si>
+    <t>Cost trends:</t>
+  </si>
+  <si>
+    <t>Assumes same rate of decline as IEA data</t>
+  </si>
+  <si>
+    <t>$/kW</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -316,6 +353,23 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -375,7 +429,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -398,6 +452,10 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -414,6 +472,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>273377</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>92201</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7D1D108D-0B02-CBE6-15FF-B4699646E697}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="180975"/>
+          <a:ext cx="6369377" cy="2444876"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -679,7 +786,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B63"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="45.81640625" customWidth="1"/>
@@ -724,224 +831,260 @@
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>28</v>
+      <c r="B10" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>29</v>
+      <c r="B11" s="7">
+        <v>2024</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>30</v>
+      <c r="B12" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>31</v>
+      <c r="B13" s="8" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>32</v>
+      <c r="B14" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>55</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>56</v>
+      <c r="A22" s="1" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>60</v>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
-        <v>33</v>
+      <c r="A27" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>35</v>
+        <v>57</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>39</v>
+      <c r="A33" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B36" t="s">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B42" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B37" s="7">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B43" s="7">
         <v>2014</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B38" t="s">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B44" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B39" s="8" t="s">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B45" s="8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B40" t="s">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B46" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A42" s="1" t="s">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A48" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B47" t="s">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B53" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B48" s="7">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B54" s="7">
         <v>2023</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B49" t="s">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B55" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B50" s="8" t="s">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B56" s="8" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A52" s="1" t="s">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A58" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A63">
+        <v>0.78452102304761584</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B7" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="B39" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="B50" r:id="rId3" xr:uid="{0EAF8239-1601-435F-A7F3-DCBE0357401E}"/>
+    <hyperlink ref="B45" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="B56" r:id="rId3" xr:uid="{0EAF8239-1601-435F-A7F3-DCBE0357401E}"/>
+    <hyperlink ref="B13" r:id="rId4" xr:uid="{0315EA59-F95F-4000-B10B-ABC8C54DF753}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="25.453125" customWidth="1"/>
@@ -950,7 +1093,7 @@
     <col min="6" max="6" width="14.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -970,7 +1113,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -989,8 +1132,12 @@
       <c r="F2">
         <v>450</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H2">
+        <f>D2*1.3</f>
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>10</v>
       </c>
@@ -1007,7 +1154,7 @@
         <v>0.74</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>12</v>
       </c>
@@ -1024,7 +1171,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="6"/>
       <c r="B5" s="6" t="s">
         <v>14</v>
@@ -1042,7 +1189,7 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1062,7 +1209,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>10</v>
       </c>
@@ -1079,7 +1226,7 @@
         <v>0.76</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>12</v>
       </c>
@@ -1096,7 +1243,7 @@
         <v>4.7E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="6"/>
       <c r="B9" s="6" t="s">
         <v>17</v>
@@ -1114,7 +1261,7 @@
         <v>8.9</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1134,7 +1281,7 @@
         <v>2670</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>10</v>
       </c>
@@ -1151,7 +1298,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>12</v>
       </c>
@@ -1168,7 +1315,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="6"/>
       <c r="B13" s="6" t="s">
         <v>17</v>
@@ -1186,8 +1333,8 @@
         <v>20.2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1207,6 +1354,86 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F673B9B9-450F-45DB-9C6D-28B16550AAC5}">
+  <dimension ref="B17:F24"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B17" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B18">
+        <v>2000</v>
+      </c>
+      <c r="C18" t="s">
+        <v>79</v>
+      </c>
+      <c r="D18" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B19" s="14">
+        <f>B18*About!A63</f>
+        <v>1569.0420460952316</v>
+      </c>
+      <c r="C19" t="s">
+        <v>79</v>
+      </c>
+      <c r="D19" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B21" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B22" s="17" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B23" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C23" s="1">
+        <v>2030</v>
+      </c>
+      <c r="D23" s="1">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B24" s="16">
+        <f>B19</f>
+        <v>1569.0420460952316</v>
+      </c>
+      <c r="C24" s="16">
+        <f>B24*'IEA Data'!E2/'IEA Data'!D2</f>
+        <v>1220.3660358518468</v>
+      </c>
+      <c r="D24" s="16">
+        <f>B24*'IEA Data'!F2/'IEA Data'!D2</f>
+        <v>784.52102304761581</v>
+      </c>
+      <c r="E24" t="s">
+        <v>85</v>
+      </c>
+      <c r="F24" t="s">
+        <v>81</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1241,7 +1468,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
@@ -1364,140 +1591,140 @@
         <v>7</v>
       </c>
       <c r="B2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,B$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.7520591062805481E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,B$1)/hours_per_year/btu_per_kwh</f>
+        <v>6.6102637228470022E-5</v>
       </c>
       <c r="C2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,C$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.7050153608740382E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,C$1)/hours_per_year/btu_per_kwh</f>
+        <v>6.4158442015867923E-5</v>
       </c>
       <c r="D2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,D$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.6579716154675392E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,D$1)/hours_per_year/btu_per_kwh</f>
+        <v>6.2214246803265824E-5</v>
       </c>
       <c r="E2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,E$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.6109278700610286E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,E$1)/hours_per_year/btu_per_kwh</f>
+        <v>6.0270051590663718E-5</v>
       </c>
       <c r="F2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,F$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.5638841246545299E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,F$1)/hours_per_year/btu_per_kwh</f>
+        <v>5.8325856378061612E-5</v>
       </c>
       <c r="G2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,G$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.5168403792480193E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,G$1)/hours_per_year/btu_per_kwh</f>
+        <v>5.6381661165459513E-5</v>
       </c>
       <c r="H2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,H$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.469796633841509E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,H$1)/hours_per_year/btu_per_kwh</f>
+        <v>5.4437465952857408E-5</v>
       </c>
       <c r="I2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,I$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.4227528884350103E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,I$1)/hours_per_year/btu_per_kwh</f>
+        <v>5.2493270740255309E-5</v>
       </c>
       <c r="J2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,J$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.3757091430284997E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,J$1)/hours_per_year/btu_per_kwh</f>
+        <v>5.054907552765321E-5</v>
       </c>
       <c r="K2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,K$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.328665397622001E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,K$1)/hours_per_year/btu_per_kwh</f>
+        <v>4.8604880315051097E-5</v>
       </c>
       <c r="L2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,L$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.2816216522154904E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,L$1)/hours_per_year/btu_per_kwh</f>
+        <v>4.6660685102449486E-5</v>
       </c>
       <c r="M2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,M$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.2345779068089914E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,M$1)/hours_per_year/btu_per_kwh</f>
+        <v>4.4716489889847387E-5</v>
       </c>
       <c r="N2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,N$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.1875341614024811E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,N$1)/hours_per_year/btu_per_kwh</f>
+        <v>4.2772294677245282E-5</v>
       </c>
       <c r="O2" s="11">
-        <f>TREND('IEA Data'!$D2:$E2,'IEA Data'!$D$15:$E$15,O$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.1404904159959821E-5</v>
+        <f>TREND('DoE Data'!$B$24:$C$24,'DoE Data'!$B$23:$C$23,O$1)/hours_per_year/btu_per_kwh</f>
+        <v>4.0828099464643176E-5</v>
       </c>
       <c r="P2" s="13">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,P$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.1022673728531968E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,P$1)/hours_per_year/btu_per_kwh</f>
+        <v>4.0099026259917448E-5</v>
       </c>
       <c r="Q2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,Q$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.0640443297104115E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,Q$1)/hours_per_year/btu_per_kwh</f>
+        <v>3.9369953055191727E-5</v>
       </c>
       <c r="R2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,R$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>2.0258212865676262E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,R$1)/hours_per_year/btu_per_kwh</f>
+        <v>3.8640879850465999E-5</v>
       </c>
       <c r="S2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,S$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.9875982434248403E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,S$1)/hours_per_year/btu_per_kwh</f>
+        <v>3.7911806645740272E-5</v>
       </c>
       <c r="T2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,T$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.949375200282055E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,T$1)/hours_per_year/btu_per_kwh</f>
+        <v>3.7182733441014544E-5</v>
       </c>
       <c r="U2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,U$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.9111521571392698E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,U$1)/hours_per_year/btu_per_kwh</f>
+        <v>3.6453660236288565E-5</v>
       </c>
       <c r="V2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,V$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.8729291139964845E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,V$1)/hours_per_year/btu_per_kwh</f>
+        <v>3.5724587031562844E-5</v>
       </c>
       <c r="W2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,W$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.8347060708536989E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,W$1)/hours_per_year/btu_per_kwh</f>
+        <v>3.4995513826837116E-5</v>
       </c>
       <c r="X2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,X$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.7964830277109136E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,X$1)/hours_per_year/btu_per_kwh</f>
+        <v>3.4266440622111389E-5</v>
       </c>
       <c r="Y2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,Y$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.7582599845681283E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,Y$1)/hours_per_year/btu_per_kwh</f>
+        <v>3.3537367417385661E-5</v>
       </c>
       <c r="Z2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,Z$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.7200369414253427E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,Z$1)/hours_per_year/btu_per_kwh</f>
+        <v>3.2808294212659689E-5</v>
       </c>
       <c r="AA2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,AA$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.6818138982825571E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,AA$1)/hours_per_year/btu_per_kwh</f>
+        <v>3.2079221007933961E-5</v>
       </c>
       <c r="AB2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,AB$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.6435908551397718E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,AB$1)/hours_per_year/btu_per_kwh</f>
+        <v>3.1350147803208234E-5</v>
       </c>
       <c r="AC2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,AC$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.6053678119969865E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,AC$1)/hours_per_year/btu_per_kwh</f>
+        <v>3.0621074598482506E-5</v>
       </c>
       <c r="AD2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,AD$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.5671447688542013E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,AD$1)/hours_per_year/btu_per_kwh</f>
+        <v>2.9892001393756778E-5</v>
       </c>
       <c r="AE2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,AE$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.5289217257114157E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,AE$1)/hours_per_year/btu_per_kwh</f>
+        <v>2.9162928189030806E-5</v>
       </c>
       <c r="AF2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,AF$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.4906986825686302E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,AF$1)/hours_per_year/btu_per_kwh</f>
+        <v>2.8433854984305078E-5</v>
       </c>
       <c r="AG2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,AG$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.4524756394258449E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,AG$1)/hours_per_year/btu_per_kwh</f>
+        <v>2.7704781779579354E-5</v>
       </c>
       <c r="AH2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,AH$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.4142525962830597E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,AH$1)/hours_per_year/btu_per_kwh</f>
+        <v>2.6975708574853626E-5</v>
       </c>
       <c r="AI2" s="11">
-        <f>TREND('IEA Data'!$E2:$F2,'IEA Data'!$E$15:$F$15,AI$1)/hours_per_year/btu_per_kwh*usd_year_conv</f>
-        <v>1.3760295531402741E-5</v>
+        <f>TREND('DoE Data'!$C$24:$D$24,'DoE Data'!$C$23:$D$23,AI$1)/hours_per_year/btu_per_kwh</f>
+        <v>2.6246635370127898E-5</v>
       </c>
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.35">
@@ -2070,139 +2297,139 @@
       </c>
       <c r="B7" s="11">
         <f>B2</f>
-        <v>2.7520591062805481E-5</v>
+        <v>6.6102637228470022E-5</v>
       </c>
       <c r="C7" s="11">
         <f t="shared" ref="C7:AI7" si="22">C2</f>
-        <v>2.7050153608740382E-5</v>
+        <v>6.4158442015867923E-5</v>
       </c>
       <c r="D7" s="11">
         <f t="shared" si="22"/>
-        <v>2.6579716154675392E-5</v>
+        <v>6.2214246803265824E-5</v>
       </c>
       <c r="E7" s="11">
         <f t="shared" si="22"/>
-        <v>2.6109278700610286E-5</v>
+        <v>6.0270051590663718E-5</v>
       </c>
       <c r="F7" s="11">
         <f t="shared" si="22"/>
-        <v>2.5638841246545299E-5</v>
+        <v>5.8325856378061612E-5</v>
       </c>
       <c r="G7" s="11">
         <f t="shared" si="22"/>
-        <v>2.5168403792480193E-5</v>
+        <v>5.6381661165459513E-5</v>
       </c>
       <c r="H7" s="11">
         <f t="shared" si="22"/>
-        <v>2.469796633841509E-5</v>
+        <v>5.4437465952857408E-5</v>
       </c>
       <c r="I7" s="11">
         <f t="shared" si="22"/>
-        <v>2.4227528884350103E-5</v>
+        <v>5.2493270740255309E-5</v>
       </c>
       <c r="J7" s="11">
         <f t="shared" si="22"/>
-        <v>2.3757091430284997E-5</v>
+        <v>5.054907552765321E-5</v>
       </c>
       <c r="K7" s="11">
         <f t="shared" si="22"/>
-        <v>2.328665397622001E-5</v>
+        <v>4.8604880315051097E-5</v>
       </c>
       <c r="L7" s="11">
         <f t="shared" si="22"/>
-        <v>2.2816216522154904E-5</v>
+        <v>4.6660685102449486E-5</v>
       </c>
       <c r="M7" s="11">
         <f t="shared" si="22"/>
-        <v>2.2345779068089914E-5</v>
+        <v>4.4716489889847387E-5</v>
       </c>
       <c r="N7" s="11">
         <f t="shared" si="22"/>
-        <v>2.1875341614024811E-5</v>
+        <v>4.2772294677245282E-5</v>
       </c>
       <c r="O7" s="11">
         <f t="shared" si="22"/>
-        <v>2.1404904159959821E-5</v>
+        <v>4.0828099464643176E-5</v>
       </c>
       <c r="P7" s="11">
         <f t="shared" si="22"/>
-        <v>2.1022673728531968E-5</v>
+        <v>4.0099026259917448E-5</v>
       </c>
       <c r="Q7" s="11">
         <f t="shared" si="22"/>
-        <v>2.0640443297104115E-5</v>
+        <v>3.9369953055191727E-5</v>
       </c>
       <c r="R7" s="11">
         <f t="shared" si="22"/>
-        <v>2.0258212865676262E-5</v>
+        <v>3.8640879850465999E-5</v>
       </c>
       <c r="S7" s="11">
         <f t="shared" si="22"/>
-        <v>1.9875982434248403E-5</v>
+        <v>3.7911806645740272E-5</v>
       </c>
       <c r="T7" s="11">
         <f t="shared" si="22"/>
-        <v>1.949375200282055E-5</v>
+        <v>3.7182733441014544E-5</v>
       </c>
       <c r="U7" s="11">
         <f t="shared" si="22"/>
-        <v>1.9111521571392698E-5</v>
+        <v>3.6453660236288565E-5</v>
       </c>
       <c r="V7" s="11">
         <f t="shared" si="22"/>
-        <v>1.8729291139964845E-5</v>
+        <v>3.5724587031562844E-5</v>
       </c>
       <c r="W7" s="11">
         <f t="shared" si="22"/>
-        <v>1.8347060708536989E-5</v>
+        <v>3.4995513826837116E-5</v>
       </c>
       <c r="X7" s="11">
         <f t="shared" si="22"/>
-        <v>1.7964830277109136E-5</v>
+        <v>3.4266440622111389E-5</v>
       </c>
       <c r="Y7" s="11">
         <f t="shared" si="22"/>
-        <v>1.7582599845681283E-5</v>
+        <v>3.3537367417385661E-5</v>
       </c>
       <c r="Z7" s="11">
         <f t="shared" si="22"/>
-        <v>1.7200369414253427E-5</v>
+        <v>3.2808294212659689E-5</v>
       </c>
       <c r="AA7" s="11">
         <f t="shared" si="22"/>
-        <v>1.6818138982825571E-5</v>
+        <v>3.2079221007933961E-5</v>
       </c>
       <c r="AB7" s="11">
         <f t="shared" si="22"/>
-        <v>1.6435908551397718E-5</v>
+        <v>3.1350147803208234E-5</v>
       </c>
       <c r="AC7" s="11">
         <f t="shared" si="22"/>
-        <v>1.6053678119969865E-5</v>
+        <v>3.0621074598482506E-5</v>
       </c>
       <c r="AD7" s="11">
         <f t="shared" si="22"/>
-        <v>1.5671447688542013E-5</v>
+        <v>2.9892001393756778E-5</v>
       </c>
       <c r="AE7" s="11">
         <f t="shared" si="22"/>
-        <v>1.5289217257114157E-5</v>
+        <v>2.9162928189030806E-5</v>
       </c>
       <c r="AF7" s="11">
         <f t="shared" si="22"/>
-        <v>1.4906986825686302E-5</v>
+        <v>2.8433854984305078E-5</v>
       </c>
       <c r="AG7" s="11">
         <f t="shared" si="22"/>
-        <v>1.4524756394258449E-5</v>
+        <v>2.7704781779579354E-5</v>
       </c>
       <c r="AH7" s="11">
         <f t="shared" si="22"/>
-        <v>1.4142525962830597E-5</v>
+        <v>2.6975708574853626E-5</v>
       </c>
       <c r="AI7" s="11">
         <f t="shared" si="22"/>
-        <v>1.3760295531402741E-5</v>
+        <v>2.6246635370127898E-5</v>
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.35">
@@ -2351,7 +2578,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
@@ -2475,139 +2702,139 @@
       </c>
       <c r="B2" s="11">
         <f>HPEC!B2*'IEA Data'!$D$4</f>
-        <v>4.1280886594208218E-7</v>
+        <v>9.9153955842705038E-7</v>
       </c>
       <c r="C2" s="11">
         <f>HPEC!C2*'IEA Data'!$D$4</f>
-        <v>4.057523041311057E-7</v>
+        <v>9.6237663023801882E-7</v>
       </c>
       <c r="D2" s="11">
         <f>HPEC!D2*'IEA Data'!$D$4</f>
-        <v>3.9869574232013086E-7</v>
+        <v>9.3321370204898737E-7</v>
       </c>
       <c r="E2" s="11">
         <f>HPEC!E2*'IEA Data'!$D$4</f>
-        <v>3.9163918050915428E-7</v>
+        <v>9.040507738599557E-7</v>
       </c>
       <c r="F2" s="11">
         <f>HPEC!F2*'IEA Data'!$D$4</f>
-        <v>3.8458261869817944E-7</v>
+        <v>8.7488784567092414E-7</v>
       </c>
       <c r="G2" s="11">
         <f>HPEC!G2*'IEA Data'!$D$4</f>
-        <v>3.7752605688720286E-7</v>
+        <v>8.4572491748189269E-7</v>
       </c>
       <c r="H2" s="11">
         <f>HPEC!H2*'IEA Data'!$D$4</f>
-        <v>3.7046949507622632E-7</v>
+        <v>8.1656198929286113E-7</v>
       </c>
       <c r="I2" s="11">
         <f>HPEC!I2*'IEA Data'!$D$4</f>
-        <v>3.6341293326525154E-7</v>
+        <v>7.8739906110382957E-7</v>
       </c>
       <c r="J2" s="11">
         <f>HPEC!J2*'IEA Data'!$D$4</f>
-        <v>3.5635637145427495E-7</v>
+        <v>7.5823613291479811E-7</v>
       </c>
       <c r="K2" s="11">
         <f>HPEC!K2*'IEA Data'!$D$4</f>
-        <v>3.4929980964330012E-7</v>
+        <v>7.2907320472576645E-7</v>
       </c>
       <c r="L2" s="11">
         <f>HPEC!L2*'IEA Data'!$D$4</f>
-        <v>3.4224324783232353E-7</v>
+        <v>6.999102765367423E-7</v>
       </c>
       <c r="M2" s="11">
         <f>HPEC!M2*'IEA Data'!$D$4</f>
-        <v>3.3518668602134869E-7</v>
+        <v>6.7074734834771074E-7</v>
       </c>
       <c r="N2" s="11">
         <f>HPEC!N2*'IEA Data'!$D$4</f>
-        <v>3.2813012421037216E-7</v>
+        <v>6.4158442015867918E-7</v>
       </c>
       <c r="O2" s="11">
         <f>HPEC!O2*'IEA Data'!$D$4</f>
-        <v>3.2107356239939732E-7</v>
+        <v>6.1242149196964762E-7</v>
       </c>
       <c r="P2" s="11">
         <f>HPEC!P2*'IEA Data'!$D$4</f>
-        <v>3.1534010592797952E-7</v>
+        <v>6.0148539389876171E-7</v>
       </c>
       <c r="Q2" s="11">
         <f>HPEC!Q2*'IEA Data'!$D$4</f>
-        <v>3.0960664945656172E-7</v>
+        <v>5.9054929582787591E-7</v>
       </c>
       <c r="R2" s="11">
         <f>HPEC!R2*'IEA Data'!$D$4</f>
-        <v>3.0387319298514391E-7</v>
+        <v>5.7961319775699E-7</v>
       </c>
       <c r="S2" s="11">
         <f>HPEC!S2*'IEA Data'!$D$4</f>
-        <v>2.9813973651372606E-7</v>
+        <v>5.6867709968610409E-7</v>
       </c>
       <c r="T2" s="11">
         <f>HPEC!T2*'IEA Data'!$D$4</f>
-        <v>2.9240628004230825E-7</v>
+        <v>5.5774100161521818E-7</v>
       </c>
       <c r="U2" s="11">
         <f>HPEC!U2*'IEA Data'!$D$4</f>
-        <v>2.8667282357089045E-7</v>
+        <v>5.4680490354432846E-7</v>
       </c>
       <c r="V2" s="11">
         <f>HPEC!V2*'IEA Data'!$D$4</f>
-        <v>2.8093936709947264E-7</v>
+        <v>5.3586880547344266E-7</v>
       </c>
       <c r="W2" s="11">
         <f>HPEC!W2*'IEA Data'!$D$4</f>
-        <v>2.7520591062805484E-7</v>
+        <v>5.2493270740255675E-7</v>
       </c>
       <c r="X2" s="11">
         <f>HPEC!X2*'IEA Data'!$D$4</f>
-        <v>2.6947245415663704E-7</v>
+        <v>5.1399660933167084E-7</v>
       </c>
       <c r="Y2" s="11">
         <f>HPEC!Y2*'IEA Data'!$D$4</f>
-        <v>2.6373899768521923E-7</v>
+        <v>5.0306051126078493E-7</v>
       </c>
       <c r="Z2" s="11">
         <f>HPEC!Z2*'IEA Data'!$D$4</f>
-        <v>2.5800554121380138E-7</v>
+        <v>4.9212441318989532E-7</v>
       </c>
       <c r="AA2" s="11">
         <f>HPEC!AA2*'IEA Data'!$D$4</f>
-        <v>2.5227208474238357E-7</v>
+        <v>4.8118831511900941E-7</v>
       </c>
       <c r="AB2" s="11">
         <f>HPEC!AB2*'IEA Data'!$D$4</f>
-        <v>2.4653862827096577E-7</v>
+        <v>4.702522170481235E-7</v>
       </c>
       <c r="AC2" s="11">
         <f>HPEC!AC2*'IEA Data'!$D$4</f>
-        <v>2.4080517179954797E-7</v>
+        <v>4.5931611897723759E-7</v>
       </c>
       <c r="AD2" s="11">
         <f>HPEC!AD2*'IEA Data'!$D$4</f>
-        <v>2.3507171532813019E-7</v>
+        <v>4.4838002090635163E-7</v>
       </c>
       <c r="AE2" s="11">
         <f>HPEC!AE2*'IEA Data'!$D$4</f>
-        <v>2.2933825885671233E-7</v>
+        <v>4.3744392283546207E-7</v>
       </c>
       <c r="AF2" s="11">
         <f>HPEC!AF2*'IEA Data'!$D$4</f>
-        <v>2.2360480238529453E-7</v>
+        <v>4.2650782476457616E-7</v>
       </c>
       <c r="AG2" s="11">
         <f>HPEC!AG2*'IEA Data'!$D$4</f>
-        <v>2.1787134591387672E-7</v>
+        <v>4.1557172669369031E-7</v>
       </c>
       <c r="AH2" s="11">
         <f>HPEC!AH2*'IEA Data'!$D$4</f>
-        <v>2.1213788944245895E-7</v>
+        <v>4.046356286228044E-7</v>
       </c>
       <c r="AI2" s="11">
         <f>HPEC!AI2*'IEA Data'!$D$4</f>
-        <v>2.0640443297104109E-7</v>
+        <v>3.9369953055191844E-7</v>
       </c>
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.35">
@@ -3180,139 +3407,139 @@
       </c>
       <c r="B7" s="11">
         <f>B2</f>
-        <v>4.1280886594208218E-7</v>
+        <v>9.9153955842705038E-7</v>
       </c>
       <c r="C7" s="11">
         <f t="shared" ref="C7:AI7" si="2">C2</f>
-        <v>4.057523041311057E-7</v>
+        <v>9.6237663023801882E-7</v>
       </c>
       <c r="D7" s="11">
         <f t="shared" si="2"/>
-        <v>3.9869574232013086E-7</v>
+        <v>9.3321370204898737E-7</v>
       </c>
       <c r="E7" s="11">
         <f t="shared" si="2"/>
-        <v>3.9163918050915428E-7</v>
+        <v>9.040507738599557E-7</v>
       </c>
       <c r="F7" s="11">
         <f t="shared" si="2"/>
-        <v>3.8458261869817944E-7</v>
+        <v>8.7488784567092414E-7</v>
       </c>
       <c r="G7" s="11">
         <f t="shared" si="2"/>
-        <v>3.7752605688720286E-7</v>
+        <v>8.4572491748189269E-7</v>
       </c>
       <c r="H7" s="11">
         <f t="shared" si="2"/>
-        <v>3.7046949507622632E-7</v>
+        <v>8.1656198929286113E-7</v>
       </c>
       <c r="I7" s="11">
         <f t="shared" si="2"/>
-        <v>3.6341293326525154E-7</v>
+        <v>7.8739906110382957E-7</v>
       </c>
       <c r="J7" s="11">
         <f t="shared" si="2"/>
-        <v>3.5635637145427495E-7</v>
+        <v>7.5823613291479811E-7</v>
       </c>
       <c r="K7" s="11">
         <f t="shared" si="2"/>
-        <v>3.4929980964330012E-7</v>
+        <v>7.2907320472576645E-7</v>
       </c>
       <c r="L7" s="11">
         <f t="shared" si="2"/>
-        <v>3.4224324783232353E-7</v>
+        <v>6.999102765367423E-7</v>
       </c>
       <c r="M7" s="11">
         <f t="shared" si="2"/>
-        <v>3.3518668602134869E-7</v>
+        <v>6.7074734834771074E-7</v>
       </c>
       <c r="N7" s="11">
         <f t="shared" si="2"/>
-        <v>3.2813012421037216E-7</v>
+        <v>6.4158442015867918E-7</v>
       </c>
       <c r="O7" s="11">
         <f t="shared" si="2"/>
-        <v>3.2107356239939732E-7</v>
+        <v>6.1242149196964762E-7</v>
       </c>
       <c r="P7" s="11">
         <f t="shared" si="2"/>
-        <v>3.1534010592797952E-7</v>
+        <v>6.0148539389876171E-7</v>
       </c>
       <c r="Q7" s="11">
         <f t="shared" si="2"/>
-        <v>3.0960664945656172E-7</v>
+        <v>5.9054929582787591E-7</v>
       </c>
       <c r="R7" s="11">
         <f t="shared" si="2"/>
-        <v>3.0387319298514391E-7</v>
+        <v>5.7961319775699E-7</v>
       </c>
       <c r="S7" s="11">
         <f t="shared" si="2"/>
-        <v>2.9813973651372606E-7</v>
+        <v>5.6867709968610409E-7</v>
       </c>
       <c r="T7" s="11">
         <f t="shared" si="2"/>
-        <v>2.9240628004230825E-7</v>
+        <v>5.5774100161521818E-7</v>
       </c>
       <c r="U7" s="11">
         <f t="shared" si="2"/>
-        <v>2.8667282357089045E-7</v>
+        <v>5.4680490354432846E-7</v>
       </c>
       <c r="V7" s="11">
         <f t="shared" si="2"/>
-        <v>2.8093936709947264E-7</v>
+        <v>5.3586880547344266E-7</v>
       </c>
       <c r="W7" s="11">
         <f t="shared" si="2"/>
-        <v>2.7520591062805484E-7</v>
+        <v>5.2493270740255675E-7</v>
       </c>
       <c r="X7" s="11">
         <f t="shared" si="2"/>
-        <v>2.6947245415663704E-7</v>
+        <v>5.1399660933167084E-7</v>
       </c>
       <c r="Y7" s="11">
         <f t="shared" si="2"/>
-        <v>2.6373899768521923E-7</v>
+        <v>5.0306051126078493E-7</v>
       </c>
       <c r="Z7" s="11">
         <f t="shared" si="2"/>
-        <v>2.5800554121380138E-7</v>
+        <v>4.9212441318989532E-7</v>
       </c>
       <c r="AA7" s="11">
         <f t="shared" si="2"/>
-        <v>2.5227208474238357E-7</v>
+        <v>4.8118831511900941E-7</v>
       </c>
       <c r="AB7" s="11">
         <f t="shared" si="2"/>
-        <v>2.4653862827096577E-7</v>
+        <v>4.702522170481235E-7</v>
       </c>
       <c r="AC7" s="11">
         <f t="shared" si="2"/>
-        <v>2.4080517179954797E-7</v>
+        <v>4.5931611897723759E-7</v>
       </c>
       <c r="AD7" s="11">
         <f t="shared" si="2"/>
-        <v>2.3507171532813019E-7</v>
+        <v>4.4838002090635163E-7</v>
       </c>
       <c r="AE7" s="11">
         <f t="shared" si="2"/>
-        <v>2.2933825885671233E-7</v>
+        <v>4.3744392283546207E-7</v>
       </c>
       <c r="AF7" s="11">
         <f t="shared" si="2"/>
-        <v>2.2360480238529453E-7</v>
+        <v>4.2650782476457616E-7</v>
       </c>
       <c r="AG7" s="11">
         <f t="shared" si="2"/>
-        <v>2.1787134591387672E-7</v>
+        <v>4.1557172669369031E-7</v>
       </c>
       <c r="AH7" s="11">
         <f t="shared" si="2"/>
-        <v>2.1213788944245895E-7</v>
+        <v>4.046356286228044E-7</v>
       </c>
       <c r="AI7" s="11">
         <f t="shared" si="2"/>
-        <v>2.0640443297104109E-7</v>
+        <v>3.9369953055191844E-7</v>
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Fix to cap/opex calculations
</commit_message>
<xml_diff>
--- a/InputData/hydgn/HPEC/Hydrogen Production Eqpt Costs.xlsx
+++ b/InputData/hydgn/HPEC/Hydrogen Production Eqpt Costs.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us-analysis\InputData\hydgn\HPEC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\hydgn\HPEC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C5DA3C0-D231-490F-9DD6-A200928C9A84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{367FBC82-7E96-48E1-B217-997B48B264DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1380" yWindow="1110" windowWidth="23535" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2880" yWindow="2505" windowWidth="21600" windowHeight="14655" tabRatio="658" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="205">
   <si>
     <t>HPEC Hydrogen Production Equipment CapEx</t>
   </si>
@@ -703,15 +703,25 @@
   <si>
     <t>Annual OpEx</t>
   </si>
+  <si>
+    <t>&lt;- resulting data</t>
+  </si>
+  <si>
+    <t>2022$/annual kg</t>
+  </si>
+  <si>
+    <t>2012$/BTU</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="171" formatCode="0.0%"/>
-    <numFmt numFmtId="181" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(&quot;$&quot;* #,##0.000_);_(&quot;$&quot;* \(#,##0.000\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -858,7 +868,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -886,21 +896,19 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -1666,13 +1674,13 @@
       <c r="F1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="H1" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
     </row>
     <row r="2" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -1693,13 +1701,13 @@
       <c r="F2">
         <v>450</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
@@ -1717,7 +1725,7 @@
       <c r="F3" s="4">
         <v>0.74</v>
       </c>
-      <c r="H3" s="23">
+      <c r="H3">
         <v>264</v>
       </c>
       <c r="I3" t="s">
@@ -1799,7 +1807,7 @@
       </c>
       <c r="H6" s="11">
         <f>HPEC!H2*'IEA Data'!B21</f>
-        <v>32.273445728952062</v>
+        <v>25.319196660549348</v>
       </c>
       <c r="J6" s="18">
         <f>J5*usd_year_conv/'IEA Data'!$B$20</f>
@@ -1996,7 +2004,7 @@
       </c>
       <c r="D21" s="18">
         <f>HPEC!I2*'IEA Data'!B21</f>
-        <v>31.120822667203726</v>
+        <v>24.414939636958092</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
@@ -2061,7 +2069,7 @@
         <f>B31/B21</f>
         <v>4.5977879999999999E-6</v>
       </c>
-      <c r="B31" s="19">
+      <c r="B31" s="18">
         <f>B23*B24*B21+B25*B26*B21</f>
         <v>0.84492756660746005</v>
       </c>
@@ -2078,7 +2086,7 @@
         <f>B32/B21</f>
         <v>4.7252268676478081E-7</v>
       </c>
-      <c r="B32" s="20">
+      <c r="B32" s="19">
         <f>HPEO!B3*B21*(1+B28)</f>
         <v>8.68346787400779E-2</v>
       </c>
@@ -2116,7 +2124,7 @@
       </c>
     </row>
     <row r="3" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="24" t="s">
         <v>134</v>
       </c>
     </row>
@@ -2204,7 +2212,7 @@
       <c r="D10">
         <v>0.15</v>
       </c>
-      <c r="F10" s="20">
+      <c r="F10" s="19">
         <f>D10*About!$A$75</f>
         <v>0.1371</v>
       </c>
@@ -2223,7 +2231,7 @@
       <c r="D11">
         <v>0.81</v>
       </c>
-      <c r="F11" s="20">
+      <c r="F11" s="19">
         <f>D11*About!$A$75</f>
         <v>0.74034000000000011</v>
       </c>
@@ -2242,7 +2250,7 @@
       <c r="D12">
         <v>0.96</v>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="19">
         <f>D12*About!$A$75</f>
         <v>0.87744</v>
       </c>
@@ -2267,7 +2275,7 @@
       </c>
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B32" s="24">
+      <c r="B32" s="22">
         <v>0.751</v>
       </c>
       <c r="C32" t="s">
@@ -2275,7 +2283,7 @@
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B33" s="24">
+      <c r="B33" s="22">
         <f>1-B32</f>
         <v>0.249</v>
       </c>
@@ -2284,7 +2292,7 @@
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B35" s="20">
+      <c r="B35" s="19">
         <f>F11*B33</f>
         <v>0.18434466000000002</v>
       </c>
@@ -2397,7 +2405,7 @@
       <c r="C44" t="s">
         <v>173</v>
       </c>
-      <c r="D44" s="27">
+      <c r="D44" s="25">
         <v>1800</v>
       </c>
       <c r="E44" t="s">
@@ -2486,7 +2494,7 @@
       <c r="C51" t="s">
         <v>173</v>
       </c>
-      <c r="D51" s="27">
+      <c r="D51" s="25">
         <v>1246</v>
       </c>
       <c r="E51" t="s">
@@ -2660,7 +2668,7 @@
       <c r="C66" t="s">
         <v>189</v>
       </c>
-      <c r="D66" s="27">
+      <c r="D66" s="25">
         <v>17069</v>
       </c>
       <c r="E66" t="s">
@@ -2703,7 +2711,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F673B9B9-450F-45DB-9C6D-28B16550AAC5}">
-  <dimension ref="A17:AE80"/>
+  <dimension ref="A17:AL83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" bestFit="1" customWidth="1"/>
@@ -2770,15 +2778,15 @@
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B24" s="31">
+      <c r="B24" s="27">
         <f>B23*$B$36/$B$43</f>
         <v>415686274.50980389</v>
       </c>
-      <c r="C24" s="31">
+      <c r="C24" s="27">
         <f t="shared" ref="C24:D24" si="0">C23*$B$36/$B$43</f>
         <v>323311546.8409586</v>
       </c>
-      <c r="D24" s="31">
+      <c r="D24" s="27">
         <f t="shared" si="0"/>
         <v>207843137.25490195</v>
       </c>
@@ -2787,49 +2795,49 @@
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B25" s="20">
+      <c r="B25" s="19">
         <f>B24/$B$35</f>
         <v>22.77733011012624</v>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="19">
         <f t="shared" ref="C25:D25" si="1">C24/$B$35</f>
         <v>17.715701196764854</v>
       </c>
-      <c r="D25" s="20">
+      <c r="D25" s="19">
         <f t="shared" si="1"/>
         <v>11.38866505506312</v>
       </c>
       <c r="E25" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="11">
-        <f>B25/'IEA Data'!$B$18*'IEA Data'!$B$19</f>
-        <v>1.6934817925744414E-4</v>
+        <f>B25/'IEA Data'!$B$18*'IEA Data'!$B$19*About!$A$72</f>
+        <v>1.328572068423011E-4</v>
       </c>
       <c r="C26" s="11">
-        <f>C25/'IEA Data'!$B$18*'IEA Data'!$B$19</f>
-        <v>1.3171525053356771E-4</v>
+        <f>C25/'IEA Data'!$B$18*'IEA Data'!$B$19*About!$A$72</f>
+        <v>1.0333338309956757E-4</v>
       </c>
       <c r="D26" s="11">
-        <f>D25/'IEA Data'!$B$18*'IEA Data'!$B$19</f>
-        <v>8.467408962872207E-5</v>
+        <f>D25/'IEA Data'!$B$18*'IEA Data'!$B$19*About!$A$72</f>
+        <v>6.6428603421150552E-5</v>
       </c>
       <c r="E26" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="31">
+      <c r="B27" s="27">
         <f>B24*5%</f>
         <v>20784313.725490198</v>
       </c>
-      <c r="C27" s="31">
+      <c r="C27" s="27">
         <f t="shared" ref="C27:D27" si="2">C24*5%</f>
         <v>16165577.34204793</v>
       </c>
-      <c r="D27" s="31">
+      <c r="D27" s="27">
         <f t="shared" si="2"/>
         <v>10392156.862745099</v>
       </c>
@@ -2841,37 +2849,37 @@
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B28" s="20">
+      <c r="B28" s="19">
         <f>B27/$B$35</f>
         <v>1.1388665055063123</v>
       </c>
-      <c r="C28" s="20">
+      <c r="C28" s="19">
         <f t="shared" ref="C28" si="3">C27/$B$35</f>
         <v>0.88578505983824274</v>
       </c>
-      <c r="D28" s="20">
+      <c r="D28" s="19">
         <f t="shared" ref="D28" si="4">D27/$B$35</f>
         <v>0.56943325275315615</v>
       </c>
       <c r="E28" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="11">
-        <f>B28/'IEA Data'!$B$18*'IEA Data'!$B$19</f>
-        <v>8.467408962872209E-6</v>
+        <f>B28/'IEA Data'!$B$18*'IEA Data'!$B$19*About!$A$72</f>
+        <v>6.6428603421150575E-6</v>
       </c>
       <c r="C29" s="11">
-        <f>C28/'IEA Data'!$B$18*'IEA Data'!$B$19</f>
-        <v>6.5857625266783848E-6</v>
+        <f>C28/'IEA Data'!$B$18*'IEA Data'!$B$19*About!$A$72</f>
+        <v>5.1666691549783778E-6</v>
       </c>
       <c r="D29" s="11">
-        <f>D28/'IEA Data'!$B$18*'IEA Data'!$B$19</f>
-        <v>4.2337044814361045E-6</v>
+        <f>D28/'IEA Data'!$B$18*'IEA Data'!$B$19*About!$A$72</f>
+        <v>3.3214301710575287E-6</v>
       </c>
       <c r="E29" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
@@ -2884,9 +2892,9 @@
         <v>124</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B33" s="25">
-        <v>1000</v>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B33" s="23">
+        <v>2000</v>
       </c>
       <c r="C33" t="s">
         <v>79</v>
@@ -2894,11 +2902,11 @@
       <c r="D33" t="s">
         <v>80</v>
       </c>
-      <c r="E33" s="25" t="s">
+      <c r="E33" s="23" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B35">
         <f>50000*365</f>
         <v>18250000</v>
@@ -2907,7 +2915,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B36">
         <v>106000</v>
       </c>
@@ -2915,7 +2923,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B37">
         <f>B35/B36</f>
         <v>172.16981132075472</v>
@@ -2924,7 +2932,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B39">
         <f>B18/B37</f>
         <v>11.616438356164384</v>
@@ -2934,7 +2942,7 @@
         <v>11.616438356164384</v>
       </c>
     </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B41">
         <f>57.5</f>
         <v>57.5</v>
@@ -2946,7 +2954,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B42">
         <v>3.3000000000000002E-2</v>
       </c>
@@ -2957,7 +2965,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B43" s="4">
         <v>0.51</v>
       </c>
@@ -2968,7 +2976,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B45">
         <f>B41*B42</f>
         <v>1.8975000000000002</v>
@@ -2980,7 +2988,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B46" s="4">
         <v>0.1</v>
       </c>
@@ -2988,10 +2996,14 @@
         <v>107</v>
       </c>
     </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B47" s="4"/>
     </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="19">
+        <f>B27/SUM(B64:AE64)/B53</f>
+        <v>0.10982736614928527</v>
+      </c>
       <c r="B48" s="4">
         <f>0.11</f>
         <v>0.11</v>
@@ -3004,7 +3016,7 @@
       </c>
     </row>
     <row r="49" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="B49" s="23">
+      <c r="B49">
         <v>40000</v>
       </c>
       <c r="C49" t="s">
@@ -3615,7 +3627,7 @@
       </c>
       <c r="B57" s="14">
         <f>B36*B33/B43</f>
-        <v>207843137.25490195</v>
+        <v>415686274.50980389</v>
       </c>
     </row>
     <row r="58" spans="1:31" x14ac:dyDescent="0.25">
@@ -3624,123 +3636,123 @@
       </c>
       <c r="B58" s="14">
         <f>5%*$B$57</f>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="C58" s="14">
         <f t="shared" ref="C58:AE58" si="7">5%*$B$57</f>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="D58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="E58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="F58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="G58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="H58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="I58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="J58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="K58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="L58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="M58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="N58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="O58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="P58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="Q58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="R58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="S58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="T58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="U58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="V58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="W58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="X58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="Y58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="Z58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="AA58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="AB58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="AC58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="AD58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="AE58" s="14">
         <f t="shared" si="7"/>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
     </row>
     <row r="59" spans="1:31" x14ac:dyDescent="0.25">
@@ -3749,119 +3761,119 @@
       </c>
       <c r="B59" s="14"/>
       <c r="C59" s="14">
-        <f>IF(C55&lt;B55,$B$57*0.11,0)</f>
+        <f t="shared" ref="C59:AE59" si="8">IF(C55&lt;B55,$B$57*0.11,0)</f>
         <v>0</v>
       </c>
       <c r="D59" s="14">
-        <f>IF(D55&lt;C55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="E59" s="14">
-        <f>IF(E55&lt;D55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F59" s="14">
-        <f>IF(F55&lt;E55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="G59" s="14">
-        <f>IF(G55&lt;F55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="H59" s="14">
-        <f>IF(H55&lt;G55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I59" s="14">
-        <f>IF(I55&lt;H55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="J59" s="14">
-        <f>IF(J55&lt;I55,$B$57*0.11,0)</f>
-        <v>22862745.098039214</v>
+        <f t="shared" si="8"/>
+        <v>45725490.196078427</v>
       </c>
       <c r="K59" s="14">
-        <f>IF(K55&lt;J55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="L59" s="14">
-        <f>IF(L55&lt;K55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M59" s="14">
-        <f>IF(M55&lt;L55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="N59" s="14">
-        <f>IF(N55&lt;M55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="O59" s="14">
-        <f>IF(O55&lt;N55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="P59" s="14">
-        <f>IF(P55&lt;O55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="Q59" s="14">
-        <f>IF(Q55&lt;P55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="R59" s="14">
-        <f>IF(R55&lt;Q55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="S59" s="14">
-        <f>IF(S55&lt;R55,$B$57*0.11,0)</f>
-        <v>22862745.098039214</v>
+        <f t="shared" si="8"/>
+        <v>45725490.196078427</v>
       </c>
       <c r="T59" s="14">
-        <f>IF(T55&lt;S55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="U59" s="14">
-        <f>IF(U55&lt;T55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="V59" s="14">
-        <f>IF(V55&lt;U55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="W59" s="14">
-        <f>IF(W55&lt;V55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="X59" s="14">
-        <f>IF(X55&lt;W55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="Y59" s="14">
-        <f>IF(Y55&lt;X55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="Z59" s="14">
-        <f>IF(Z55&lt;Y55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="AA59" s="14">
-        <f>IF(AA55&lt;Z55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="AB59" s="14">
-        <f>IF(AB55&lt;AA55,$B$57*0.11,0)</f>
-        <v>22862745.098039214</v>
+        <f t="shared" si="8"/>
+        <v>45725490.196078427</v>
       </c>
       <c r="AC59" s="14">
-        <f>IF(AC55&lt;AB55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="AD59" s="14">
-        <f>IF(AD55&lt;AC55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="AE59" s="14">
-        <f>IF(AE55&lt;AD55,$B$57*0.11,0)</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -3903,123 +3915,123 @@
       </c>
       <c r="B61" s="14">
         <f>SUM(B56:B59)/(1+$B$46)^(B52-1)</f>
-        <v>252864669.11764705</v>
+        <v>471099963.2352941</v>
       </c>
       <c r="C61" s="14">
-        <f t="shared" ref="C61:AE61" si="8">SUM(C56:C59)/(1+$B$46)^(C52-1)</f>
-        <v>40928665.32976827</v>
+        <f t="shared" ref="C61:AE61" si="9">SUM(C56:C59)/(1+$B$46)^(C52-1)</f>
+        <v>50376080.659536541</v>
       </c>
       <c r="D61" s="14">
-        <f t="shared" si="8"/>
-        <v>37207877.572516605</v>
+        <f t="shared" si="9"/>
+        <v>45796436.963215031</v>
       </c>
       <c r="E61" s="14">
-        <f t="shared" si="8"/>
-        <v>33825343.247742362</v>
+        <f t="shared" si="9"/>
+        <v>41633124.512013659</v>
       </c>
       <c r="F61" s="14">
-        <f t="shared" si="8"/>
-        <v>30750312.04340215</v>
+        <f t="shared" si="9"/>
+        <v>37848295.010921508</v>
       </c>
       <c r="G61" s="14">
-        <f t="shared" si="8"/>
-        <v>27954829.130365588</v>
+        <f t="shared" si="9"/>
+        <v>34407540.91901955</v>
       </c>
       <c r="H61" s="14">
-        <f t="shared" si="8"/>
-        <v>25413481.027605075</v>
+        <f t="shared" si="9"/>
+        <v>31279582.653654136</v>
       </c>
       <c r="I61" s="14">
-        <f t="shared" si="8"/>
-        <v>23103164.570550065</v>
+        <f t="shared" si="9"/>
+        <v>28435984.230594665</v>
       </c>
       <c r="J61" s="14">
-        <f t="shared" si="8"/>
-        <v>31668516.202407438</v>
+        <f t="shared" si="9"/>
+        <v>47182173.395264447</v>
       </c>
       <c r="K61" s="14">
-        <f t="shared" si="8"/>
-        <v>19093524.438471131</v>
+        <f t="shared" si="9"/>
+        <v>23500813.413714599</v>
       </c>
       <c r="L61" s="14">
-        <f t="shared" si="8"/>
-        <v>17357749.489519205</v>
+        <f t="shared" si="9"/>
+        <v>21364375.830649633</v>
       </c>
       <c r="M61" s="14">
-        <f t="shared" si="8"/>
-        <v>15779772.263199277</v>
+        <f t="shared" si="9"/>
+        <v>19422159.846045118</v>
       </c>
       <c r="N61" s="14">
-        <f t="shared" si="8"/>
-        <v>14345247.511999343</v>
+        <f t="shared" si="9"/>
+        <v>17656508.950950108</v>
       </c>
       <c r="O61" s="14">
-        <f t="shared" si="8"/>
-        <v>13041134.101817584</v>
+        <f t="shared" si="9"/>
+        <v>16051371.773591006</v>
       </c>
       <c r="P61" s="14">
-        <f t="shared" si="8"/>
-        <v>11855576.456197802</v>
+        <f t="shared" si="9"/>
+        <v>14592156.157810003</v>
       </c>
       <c r="Q61" s="14">
-        <f t="shared" si="8"/>
-        <v>10777796.778361637</v>
+        <f t="shared" si="9"/>
+        <v>13265596.507100003</v>
       </c>
       <c r="R61" s="14">
-        <f t="shared" si="8"/>
-        <v>9797997.0712378528</v>
+        <f t="shared" si="9"/>
+        <v>12059633.18827273</v>
       </c>
       <c r="S61" s="14">
-        <f t="shared" si="8"/>
-        <v>13430542.298831437</v>
+        <f t="shared" si="9"/>
+        <v>20009847.366569262</v>
       </c>
       <c r="T61" s="14">
-        <f t="shared" si="8"/>
-        <v>8097518.2406924395</v>
+        <f t="shared" si="9"/>
+        <v>9966638.9985725023</v>
       </c>
       <c r="U61" s="14">
-        <f t="shared" si="8"/>
-        <v>7361380.2188113062</v>
+        <f t="shared" si="9"/>
+        <v>9060580.9077931829</v>
       </c>
       <c r="V61" s="14">
-        <f t="shared" si="8"/>
-        <v>6692163.8352830065</v>
+        <f t="shared" si="9"/>
+        <v>8236891.734357439</v>
       </c>
       <c r="W61" s="14">
-        <f t="shared" si="8"/>
-        <v>6083785.3048027325</v>
+        <f t="shared" si="9"/>
+        <v>7488083.3948703976</v>
       </c>
       <c r="X61" s="14">
-        <f t="shared" si="8"/>
-        <v>5530713.9134570286</v>
+        <f t="shared" si="9"/>
+        <v>6807348.5407912703</v>
       </c>
       <c r="Y61" s="14">
-        <f t="shared" si="8"/>
-        <v>5027921.739506389</v>
+        <f t="shared" si="9"/>
+        <v>6188498.6734466087</v>
       </c>
       <c r="Z61" s="14">
-        <f t="shared" si="8"/>
-        <v>4570837.945005809</v>
+        <f t="shared" si="9"/>
+        <v>5625907.884951463</v>
       </c>
       <c r="AA61" s="14">
-        <f t="shared" si="8"/>
-        <v>4155307.2227325528</v>
+        <f t="shared" si="9"/>
+        <v>5114461.7135922378</v>
       </c>
       <c r="AB61" s="14">
-        <f t="shared" si="8"/>
-        <v>5695861.0023853276</v>
+        <f t="shared" si="9"/>
+        <v>8486128.6121589579</v>
       </c>
       <c r="AC61" s="14">
-        <f t="shared" si="8"/>
-        <v>3434138.2006054148</v>
+        <f t="shared" si="9"/>
+        <v>4226827.8624729235</v>
       </c>
       <c r="AD61" s="14">
-        <f t="shared" si="8"/>
-        <v>3121943.8187321955</v>
+        <f t="shared" si="9"/>
+        <v>3842570.7840662939</v>
       </c>
       <c r="AE61" s="14">
-        <f t="shared" si="8"/>
-        <v>2838130.7443019957</v>
+        <f t="shared" si="9"/>
+        <v>3493246.1673329943</v>
       </c>
     </row>
     <row r="62" spans="1:31" x14ac:dyDescent="0.25">
@@ -4028,122 +4040,122 @@
       </c>
       <c r="B62" s="14">
         <f>(B57+B59)/(1+$B$46)^(B52-1)</f>
-        <v>207843137.25490195</v>
+        <v>415686274.50980389</v>
       </c>
       <c r="C62">
-        <f t="shared" ref="C62:AE62" si="9">(C57+C59)/(1+$B$46)^(C52-1)</f>
+        <f t="shared" ref="C62:AE62" si="10">(C57+C59)/(1+$B$46)^(C52-1)</f>
         <v>0</v>
       </c>
       <c r="D62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="E62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="G62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="H62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="I62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J62">
-        <f t="shared" si="9"/>
-        <v>10665639.320089193</v>
+        <f t="shared" si="10"/>
+        <v>21331278.640178386</v>
       </c>
       <c r="K62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="L62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="M62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="N62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="O62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="P62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="Q62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="R62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="S62">
-        <f t="shared" si="9"/>
-        <v>4523272.2340697534</v>
+        <f t="shared" si="10"/>
+        <v>9046544.4681395069</v>
       </c>
       <c r="T62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="V62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="W62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="X62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="Y62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="Z62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AA62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AB62">
-        <f t="shared" si="9"/>
-        <v>1918308.9817193702</v>
+        <f t="shared" si="10"/>
+        <v>3836617.9634387405</v>
       </c>
       <c r="AC62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AD62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AE62">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -4153,123 +4165,123 @@
       </c>
       <c r="B63">
         <f>B58/(1+$B$46)^(B52-1)</f>
-        <v>10392156.862745099</v>
+        <v>20784313.725490198</v>
       </c>
       <c r="C63">
-        <f t="shared" ref="C63:AE63" si="10">C58/(1+$B$46)^(C52-1)</f>
-        <v>9447415.3297682703</v>
+        <f t="shared" ref="C63:AE63" si="11">C58/(1+$B$46)^(C52-1)</f>
+        <v>18894830.659536541</v>
       </c>
       <c r="D63">
-        <f t="shared" si="10"/>
-        <v>8588559.3906984273</v>
+        <f t="shared" si="11"/>
+        <v>17177118.781396855</v>
       </c>
       <c r="E63">
-        <f t="shared" si="10"/>
-        <v>7807781.2642712966</v>
+        <f t="shared" si="11"/>
+        <v>15615562.528542593</v>
       </c>
       <c r="F63">
-        <f t="shared" si="10"/>
-        <v>7097982.9675193606</v>
+        <f t="shared" si="11"/>
+        <v>14195965.935038721</v>
       </c>
       <c r="G63">
-        <f t="shared" si="10"/>
-        <v>6452711.7886539642</v>
+        <f t="shared" si="11"/>
+        <v>12905423.577307928</v>
       </c>
       <c r="H63">
-        <f t="shared" si="10"/>
-        <v>5866101.6260490576</v>
+        <f t="shared" si="11"/>
+        <v>11732203.252098115</v>
       </c>
       <c r="I63">
-        <f t="shared" si="10"/>
-        <v>5332819.6600445965</v>
+        <f t="shared" si="11"/>
+        <v>10665639.320089193</v>
       </c>
       <c r="J63">
-        <f t="shared" si="10"/>
-        <v>4848017.8727678154</v>
+        <f t="shared" si="11"/>
+        <v>9696035.7455356307</v>
       </c>
       <c r="K63">
-        <f t="shared" si="10"/>
-        <v>4407288.9752434688</v>
+        <f t="shared" si="11"/>
+        <v>8814577.9504869375</v>
       </c>
       <c r="L63">
-        <f t="shared" si="10"/>
-        <v>4006626.3411304252</v>
+        <f t="shared" si="11"/>
+        <v>8013252.6822608504</v>
       </c>
       <c r="M63">
-        <f t="shared" si="10"/>
-        <v>3642387.5828458406</v>
+        <f t="shared" si="11"/>
+        <v>7284775.1656916812</v>
       </c>
       <c r="N63">
-        <f t="shared" si="10"/>
-        <v>3311261.4389507645</v>
+        <f t="shared" si="11"/>
+        <v>6622522.877901529</v>
       </c>
       <c r="O63">
-        <f t="shared" si="10"/>
-        <v>3010237.671773422</v>
+        <f t="shared" si="11"/>
+        <v>6020475.3435468441</v>
       </c>
       <c r="P63">
-        <f t="shared" si="10"/>
-        <v>2736579.7016122015</v>
+        <f t="shared" si="11"/>
+        <v>5473159.403224403</v>
       </c>
       <c r="Q63">
-        <f t="shared" si="10"/>
-        <v>2487799.7287383648</v>
+        <f t="shared" si="11"/>
+        <v>4975599.4574767295</v>
       </c>
       <c r="R63">
-        <f t="shared" si="10"/>
-        <v>2261636.1170348772</v>
+        <f t="shared" si="11"/>
+        <v>4523272.2340697544</v>
       </c>
       <c r="S63">
-        <f t="shared" si="10"/>
-        <v>2056032.8336680701</v>
+        <f t="shared" si="11"/>
+        <v>4112065.6673361403</v>
       </c>
       <c r="T63">
-        <f t="shared" si="10"/>
-        <v>1869120.7578800635</v>
+        <f t="shared" si="11"/>
+        <v>3738241.515760127</v>
       </c>
       <c r="U63">
-        <f t="shared" si="10"/>
-        <v>1699200.6889818755</v>
+        <f t="shared" si="11"/>
+        <v>3398401.3779637511</v>
       </c>
       <c r="V63">
-        <f t="shared" si="10"/>
-        <v>1544727.8990744324</v>
+        <f t="shared" si="11"/>
+        <v>3089455.7981488649</v>
       </c>
       <c r="W63">
-        <f t="shared" si="10"/>
-        <v>1404298.0900676658</v>
+        <f t="shared" si="11"/>
+        <v>2808596.1801353316</v>
       </c>
       <c r="X63">
-        <f t="shared" si="10"/>
-        <v>1276634.6273342413</v>
+        <f t="shared" si="11"/>
+        <v>2553269.2546684826</v>
       </c>
       <c r="Y63">
-        <f t="shared" si="10"/>
-        <v>1160576.9339402192</v>
+        <f t="shared" si="11"/>
+        <v>2321153.8678804385</v>
       </c>
       <c r="Z63">
-        <f t="shared" si="10"/>
-        <v>1055069.939945654</v>
+        <f t="shared" si="11"/>
+        <v>2110139.879891308</v>
       </c>
       <c r="AA63">
-        <f t="shared" si="10"/>
-        <v>959154.49085968535</v>
+        <f t="shared" si="11"/>
+        <v>1918308.9817193707</v>
       </c>
       <c r="AB63">
-        <f t="shared" si="10"/>
-        <v>871958.62805425934</v>
+        <f t="shared" si="11"/>
+        <v>1743917.2561085187</v>
       </c>
       <c r="AC63">
-        <f t="shared" si="10"/>
-        <v>792689.66186750832</v>
+        <f t="shared" si="11"/>
+        <v>1585379.3237350166</v>
       </c>
       <c r="AD63">
-        <f t="shared" si="10"/>
-        <v>720626.96533409855</v>
+        <f t="shared" si="11"/>
+        <v>1441253.9306681971</v>
       </c>
       <c r="AE63">
-        <f t="shared" si="10"/>
-        <v>655115.42303099867</v>
+        <f t="shared" si="11"/>
+        <v>1310230.8460619973</v>
       </c>
     </row>
     <row r="64" spans="1:31" x14ac:dyDescent="0.25">
@@ -4278,160 +4290,174 @@
         <v>1</v>
       </c>
       <c r="C64">
-        <f t="shared" ref="C64:AE64" si="11">1/((1+$B$46)^(C52-1))</f>
+        <f t="shared" ref="C64:AE64" si="12">1/((1+$B$46)^(C52-1))</f>
         <v>0.90909090909090906</v>
       </c>
       <c r="D64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.82644628099173545</v>
       </c>
       <c r="E64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.75131480090157754</v>
       </c>
       <c r="F64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.68301345536507052</v>
       </c>
       <c r="G64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.62092132305915493</v>
       </c>
       <c r="H64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.56447393005377722</v>
       </c>
       <c r="I64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.51315811823070645</v>
       </c>
       <c r="J64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.46650738020973315</v>
       </c>
       <c r="K64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.42409761837248466</v>
       </c>
       <c r="L64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.38554328942953148</v>
       </c>
       <c r="M64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.3504938994813922</v>
       </c>
       <c r="N64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.31863081771035656</v>
       </c>
       <c r="O64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.28966437973668779</v>
       </c>
       <c r="P64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.26333125430607973</v>
       </c>
       <c r="Q64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.23939204936916339</v>
       </c>
       <c r="R64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.21762913579014853</v>
       </c>
       <c r="S64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.19784466890013502</v>
       </c>
       <c r="T64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.17985878990921364</v>
       </c>
       <c r="U64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.16350799082655781</v>
       </c>
       <c r="V64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.14864362802414349</v>
       </c>
       <c r="W64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.13513057093103953</v>
       </c>
       <c r="X64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.12284597357367227</v>
       </c>
       <c r="Y64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.11167815779424752</v>
       </c>
       <c r="Z64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.10152559799477048</v>
       </c>
       <c r="AA64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>9.2295998177064048E-2</v>
       </c>
       <c r="AB64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>8.3905452888240042E-2</v>
       </c>
       <c r="AC64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>7.6277684443854576E-2</v>
       </c>
       <c r="AD64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>6.9343349494413245E-2</v>
       </c>
       <c r="AE64">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>6.3039408631284766E-2</v>
       </c>
     </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:38" x14ac:dyDescent="0.25">
       <c r="C65" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B66">
         <f>SUM(B61:AE61)/SUM(B64:AE64)/B53</f>
-        <v>3.6556039799564948</v>
+        <v>5.4137079599129887</v>
       </c>
       <c r="C66" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="67" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B67">
+    <row r="67" spans="2:38" x14ac:dyDescent="0.25">
+      <c r="B67" s="28">
         <f>SUM(B62:AE62)/SUM(B64:AE64)/B53</f>
-        <v>1.1886707272033381</v>
+        <v>2.3773414544066762</v>
       </c>
       <c r="C67" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="68" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B68">
+      <c r="E67" s="23" t="s">
+        <v>202</v>
+      </c>
+      <c r="G67">
+        <f>SUM(B63:J63)/SUM(B64:J64)</f>
+        <v>20784313.72549019</v>
+      </c>
+    </row>
+    <row r="68" spans="2:38" x14ac:dyDescent="0.25">
+      <c r="B68" s="28">
         <f>SUM(B63:AE63)/SUM(B64:AE64)/B53</f>
-        <v>0.56943325275315604</v>
+        <v>1.1388665055063121</v>
       </c>
       <c r="C68" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="70" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="E68" s="23" t="s">
+        <v>202</v>
+      </c>
+      <c r="H68">
+        <f>SUM(B64:AE64)</f>
+        <v>10.369605913687147</v>
+      </c>
+    </row>
+    <row r="70" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B70" s="15" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="71" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B71">
         <v>2024</v>
       </c>
@@ -4442,9 +4468,9 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="72" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B72">
-        <v>2.1965473229857051</v>
+        <v>2.19654732298571</v>
       </c>
       <c r="C72">
         <v>1.7089138172828786</v>
@@ -4455,11 +4481,12 @@
       <c r="E72" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="73" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="G72" s="29"/>
+    </row>
+    <row r="73" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B73">
         <f>B72*About!$A$72</f>
-        <v>1.7232375530012471</v>
+        <v>1.7232375530012511</v>
       </c>
       <c r="C73">
         <f>C72*About!$A$72</f>
@@ -4473,10 +4500,10 @@
         <v>126</v>
       </c>
     </row>
-    <row r="74" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B74" s="11">
         <f>B73/'IEA Data'!$B$18*'IEA Data'!$B$19</f>
-        <v>1.2812175115250908E-5</v>
+        <v>1.2812175115250939E-5</v>
       </c>
       <c r="C74" s="11">
         <f>C73/'IEA Data'!$B$18*'IEA Data'!$B$19</f>
@@ -4490,12 +4517,12 @@
         <v>127</v>
       </c>
     </row>
-    <row r="76" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B76" s="15" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="77" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B77">
         <v>2024</v>
       </c>
@@ -4506,7 +4533,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="78" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B78">
         <v>1.1388665055063121</v>
       </c>
@@ -4519,8 +4546,47 @@
       <c r="E78" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="79" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="I78">
+        <v>60</v>
+      </c>
+      <c r="J78">
+        <f>I78*J79/I79</f>
+        <v>54.545454545454547</v>
+      </c>
+      <c r="K78">
+        <f t="shared" ref="K78:R78" si="13">J78*K79/J79</f>
+        <v>49.586776859504127</v>
+      </c>
+      <c r="L78">
+        <f t="shared" si="13"/>
+        <v>45.078888054094648</v>
+      </c>
+      <c r="M78">
+        <f t="shared" si="13"/>
+        <v>40.98080732190423</v>
+      </c>
+      <c r="N78">
+        <f t="shared" si="13"/>
+        <v>37.255279383549293</v>
+      </c>
+      <c r="O78">
+        <f t="shared" si="13"/>
+        <v>33.868435803226632</v>
+      </c>
+      <c r="P78">
+        <f t="shared" si="13"/>
+        <v>30.789487093842389</v>
+      </c>
+      <c r="Q78">
+        <f t="shared" si="13"/>
+        <v>27.990442812583989</v>
+      </c>
+      <c r="R78">
+        <f t="shared" si="13"/>
+        <v>25.44585710234908</v>
+      </c>
+    </row>
+    <row r="79" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B79">
         <f>B78*About!$A$72</f>
         <v>0.89346471601447519</v>
@@ -4536,8 +4602,98 @@
       <c r="E79" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="80" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="I79">
+        <v>1</v>
+      </c>
+      <c r="J79">
+        <v>0.90909090909090906</v>
+      </c>
+      <c r="K79">
+        <v>0.82644628099173545</v>
+      </c>
+      <c r="L79">
+        <v>0.75131480090157754</v>
+      </c>
+      <c r="M79">
+        <v>0.68301345536507052</v>
+      </c>
+      <c r="N79">
+        <v>0.62092132305915493</v>
+      </c>
+      <c r="O79">
+        <v>0.56447393005377722</v>
+      </c>
+      <c r="P79">
+        <v>0.51315811823070645</v>
+      </c>
+      <c r="Q79">
+        <v>0.46650738020973315</v>
+      </c>
+      <c r="R79">
+        <v>0.42409761837248466</v>
+      </c>
+      <c r="S79">
+        <v>0.38554328942953148</v>
+      </c>
+      <c r="T79">
+        <v>0.3504938994813922</v>
+      </c>
+      <c r="U79">
+        <v>0.31863081771035656</v>
+      </c>
+      <c r="V79">
+        <v>0.28966437973668779</v>
+      </c>
+      <c r="W79">
+        <v>0.26333125430607973</v>
+      </c>
+      <c r="X79">
+        <v>0.23939204936916339</v>
+      </c>
+      <c r="Y79">
+        <v>0.21762913579014853</v>
+      </c>
+      <c r="Z79">
+        <v>0.19784466890013502</v>
+      </c>
+      <c r="AA79">
+        <v>0.17985878990921364</v>
+      </c>
+      <c r="AB79">
+        <v>0.16350799082655781</v>
+      </c>
+      <c r="AC79">
+        <v>0.14864362802414349</v>
+      </c>
+      <c r="AD79">
+        <v>0.13513057093103953</v>
+      </c>
+      <c r="AE79">
+        <v>0.12284597357367227</v>
+      </c>
+      <c r="AF79">
+        <v>0.11167815779424752</v>
+      </c>
+      <c r="AG79">
+        <v>0.10152559799477048</v>
+      </c>
+      <c r="AH79">
+        <v>9.2295998177064048E-2</v>
+      </c>
+      <c r="AI79">
+        <v>8.3905452888240042E-2</v>
+      </c>
+      <c r="AJ79">
+        <v>7.6277684443854576E-2</v>
+      </c>
+      <c r="AK79">
+        <v>6.9343349494413245E-2</v>
+      </c>
+      <c r="AL79">
+        <v>6.3039408631284766E-2</v>
+      </c>
+    </row>
+    <row r="80" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B80" s="11">
         <f>B79/'IEA Data'!$B$18*'IEA Data'!$B$19</f>
         <v>6.6428603421150575E-6</v>
@@ -4552,6 +4708,22 @@
       </c>
       <c r="E80" t="s">
         <v>127</v>
+      </c>
+      <c r="I80">
+        <f>SUM(I78:R78)/SUM(I79:AL79)</f>
+        <v>39.108663564660922</v>
+      </c>
+    </row>
+    <row r="82" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I82">
+        <f>SUM(I79:R79)/SUM(I79:AL79)</f>
+        <v>0.65181105941101536</v>
+      </c>
+    </row>
+    <row r="83" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I83">
+        <f>I82*I78</f>
+        <v>39.108663564660922</v>
       </c>
     </row>
   </sheetData>
@@ -4721,139 +4893,139 @@
       </c>
       <c r="B2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,B$1)</f>
-        <v>2.1325326276863329E-4</v>
+        <v>1.6730166787549267E-4</v>
       </c>
       <c r="C2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,C$1)</f>
-        <v>2.0698110798132198E-4</v>
+        <v>1.6238103058503588E-4</v>
       </c>
       <c r="D2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,D$1)</f>
-        <v>2.0070895319400893E-4</v>
+        <v>1.5746039329458082E-4</v>
       </c>
       <c r="E2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,E$1)</f>
-        <v>1.9443679840669588E-4</v>
+        <v>1.5253975600412577E-4</v>
       </c>
       <c r="F2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,F$1)</f>
-        <v>1.8816464361938283E-4</v>
+        <v>1.4761911871366898E-4</v>
       </c>
       <c r="G2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,G$1)</f>
-        <v>1.8189248883206978E-4</v>
+        <v>1.4269848142321392E-4</v>
       </c>
       <c r="H2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,H$1)</f>
-        <v>1.7562033404475846E-4</v>
+        <v>1.3777784413275887E-4</v>
       </c>
       <c r="I2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,I$1)</f>
-        <v>1.6934817925744541E-4</v>
+        <v>1.3285720684230208E-4</v>
       </c>
       <c r="J2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,J$1)</f>
-        <v>1.6307602447013236E-4</v>
+        <v>1.2793656955184703E-4</v>
       </c>
       <c r="K2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,K$1)</f>
-        <v>1.5680386968281931E-4</v>
+        <v>1.2301593226139197E-4</v>
       </c>
       <c r="L2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,L$1)</f>
-        <v>1.5053171489550626E-4</v>
+        <v>1.1809529497093518E-4</v>
       </c>
       <c r="M2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,M$1)</f>
-        <v>1.4425956010819321E-4</v>
+        <v>1.1317465768048013E-4</v>
       </c>
       <c r="N2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,N$1)</f>
-        <v>1.379874053208819E-4</v>
+        <v>1.0825402039002507E-4</v>
       </c>
       <c r="O2" s="11">
         <f>TREND('DoE Data'!$B$26:$C$26,'DoE Data'!$B$22:$C$22,O$1)</f>
-        <v>1.3171525053356885E-4</v>
+        <v>1.0333338309957002E-4</v>
       </c>
       <c r="P2" s="13">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,P$1)</f>
-        <v>1.2936319248832515E-4</v>
+        <v>1.0148814411564677E-4</v>
       </c>
       <c r="Q2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,Q$1)</f>
-        <v>1.2701113444308319E-4</v>
+        <v>9.9642905131726127E-5</v>
       </c>
       <c r="R2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,R$1)</f>
-        <v>1.2465907639784123E-4</v>
+        <v>9.7797666147805048E-5</v>
       </c>
       <c r="S2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,S$1)</f>
-        <v>1.2230701835259841E-4</v>
+        <v>9.5952427163884402E-5</v>
       </c>
       <c r="T2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,T$1)</f>
-        <v>1.1995496030735645E-4</v>
+        <v>9.4107188179963323E-5</v>
       </c>
       <c r="U2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,U$1)</f>
-        <v>1.1760290226211362E-4</v>
+        <v>9.2261949196042678E-5</v>
       </c>
       <c r="V2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,V$1)</f>
-        <v>1.1525084421687166E-4</v>
+        <v>9.0416710212121599E-5</v>
       </c>
       <c r="W2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,W$1)</f>
-        <v>1.128987861716297E-4</v>
+        <v>8.8571471228200954E-5</v>
       </c>
       <c r="X2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,X$1)</f>
-        <v>1.1054672812638687E-4</v>
+        <v>8.6726232244279874E-5</v>
       </c>
       <c r="Y2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,Y$1)</f>
-        <v>1.0819467008114491E-4</v>
+        <v>8.4880993260359229E-5</v>
       </c>
       <c r="Z2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,Z$1)</f>
-        <v>1.0584261203590295E-4</v>
+        <v>8.303575427643815E-5</v>
       </c>
       <c r="AA2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,AA$1)</f>
-        <v>1.0349055399066012E-4</v>
+        <v>8.1190515292517505E-5</v>
       </c>
       <c r="AB2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,AB$1)</f>
-        <v>1.0113849594541816E-4</v>
+        <v>7.9345276308596425E-5</v>
       </c>
       <c r="AC2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,AC$1)</f>
-        <v>9.8786437900175335E-5</v>
+        <v>7.750003732467578E-5</v>
       </c>
       <c r="AD2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,AD$1)</f>
-        <v>9.6434379854933375E-5</v>
+        <v>7.5654798340754701E-5</v>
       </c>
       <c r="AE2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,AE$1)</f>
-        <v>9.4082321809691415E-5</v>
+        <v>7.3809559356834056E-5</v>
       </c>
       <c r="AF2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,AF$1)</f>
-        <v>9.1730263764448587E-5</v>
+        <v>7.1964320372912977E-5</v>
       </c>
       <c r="AG2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,AG$1)</f>
-        <v>8.9378205719206627E-5</v>
+        <v>7.0119081388992331E-5</v>
       </c>
       <c r="AH2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,AH$1)</f>
-        <v>8.7026147673964667E-5</v>
+        <v>6.8273842405071686E-5</v>
       </c>
       <c r="AI2" s="11">
         <f>TREND('DoE Data'!$C$26:$D$26,'DoE Data'!$C$22:$D$22,AI$1)</f>
-        <v>8.4674089628721839E-5</v>
+        <v>6.6428603421150607E-5</v>
       </c>
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.25">
@@ -5335,7 +5507,7 @@
         <f t="shared" si="21"/>
         <v>6.8364984468095934E-6</v>
       </c>
-      <c r="O6" s="29">
+      <c r="O6">
         <f t="shared" si="21"/>
         <v>6.8364984468095934E-6</v>
       </c>
@@ -5426,139 +5598,139 @@
       </c>
       <c r="B7" s="11">
         <f>B2</f>
-        <v>2.1325326276863329E-4</v>
+        <v>1.6730166787549267E-4</v>
       </c>
       <c r="C7" s="11">
         <f t="shared" ref="C7:AI7" si="23">C2</f>
-        <v>2.0698110798132198E-4</v>
+        <v>1.6238103058503588E-4</v>
       </c>
       <c r="D7" s="11">
         <f t="shared" si="23"/>
-        <v>2.0070895319400893E-4</v>
+        <v>1.5746039329458082E-4</v>
       </c>
       <c r="E7" s="11">
         <f t="shared" si="23"/>
-        <v>1.9443679840669588E-4</v>
+        <v>1.5253975600412577E-4</v>
       </c>
       <c r="F7" s="11">
         <f t="shared" si="23"/>
-        <v>1.8816464361938283E-4</v>
+        <v>1.4761911871366898E-4</v>
       </c>
       <c r="G7" s="11">
         <f t="shared" si="23"/>
-        <v>1.8189248883206978E-4</v>
+        <v>1.4269848142321392E-4</v>
       </c>
       <c r="H7" s="11">
         <f t="shared" si="23"/>
-        <v>1.7562033404475846E-4</v>
+        <v>1.3777784413275887E-4</v>
       </c>
       <c r="I7" s="11">
         <f t="shared" si="23"/>
-        <v>1.6934817925744541E-4</v>
+        <v>1.3285720684230208E-4</v>
       </c>
       <c r="J7" s="11">
         <f t="shared" si="23"/>
-        <v>1.6307602447013236E-4</v>
+        <v>1.2793656955184703E-4</v>
       </c>
       <c r="K7" s="11">
         <f t="shared" si="23"/>
-        <v>1.5680386968281931E-4</v>
+        <v>1.2301593226139197E-4</v>
       </c>
       <c r="L7" s="11">
         <f t="shared" si="23"/>
-        <v>1.5053171489550626E-4</v>
+        <v>1.1809529497093518E-4</v>
       </c>
       <c r="M7" s="11">
         <f t="shared" si="23"/>
-        <v>1.4425956010819321E-4</v>
-      </c>
-      <c r="N7" s="28">
+        <v>1.1317465768048013E-4</v>
+      </c>
+      <c r="N7" s="11">
         <f t="shared" si="23"/>
-        <v>1.379874053208819E-4</v>
-      </c>
-      <c r="O7" s="30">
+        <v>1.0825402039002507E-4</v>
+      </c>
+      <c r="O7" s="26">
         <f t="shared" si="23"/>
-        <v>1.3171525053356885E-4</v>
+        <v>1.0333338309957002E-4</v>
       </c>
       <c r="P7" s="11">
         <f t="shared" si="23"/>
-        <v>1.2936319248832515E-4</v>
+        <v>1.0148814411564677E-4</v>
       </c>
       <c r="Q7" s="11">
         <f t="shared" si="23"/>
-        <v>1.2701113444308319E-4</v>
+        <v>9.9642905131726127E-5</v>
       </c>
       <c r="R7" s="11">
         <f t="shared" si="23"/>
-        <v>1.2465907639784123E-4</v>
+        <v>9.7797666147805048E-5</v>
       </c>
       <c r="S7" s="11">
         <f t="shared" si="23"/>
-        <v>1.2230701835259841E-4</v>
+        <v>9.5952427163884402E-5</v>
       </c>
       <c r="T7" s="11">
         <f t="shared" si="23"/>
-        <v>1.1995496030735645E-4</v>
+        <v>9.4107188179963323E-5</v>
       </c>
       <c r="U7" s="11">
         <f t="shared" si="23"/>
-        <v>1.1760290226211362E-4</v>
+        <v>9.2261949196042678E-5</v>
       </c>
       <c r="V7" s="11">
         <f t="shared" si="23"/>
-        <v>1.1525084421687166E-4</v>
+        <v>9.0416710212121599E-5</v>
       </c>
       <c r="W7" s="11">
         <f t="shared" si="23"/>
-        <v>1.128987861716297E-4</v>
+        <v>8.8571471228200954E-5</v>
       </c>
       <c r="X7" s="11">
         <f t="shared" si="23"/>
-        <v>1.1054672812638687E-4</v>
+        <v>8.6726232244279874E-5</v>
       </c>
       <c r="Y7" s="11">
         <f t="shared" si="23"/>
-        <v>1.0819467008114491E-4</v>
+        <v>8.4880993260359229E-5</v>
       </c>
       <c r="Z7" s="11">
         <f t="shared" si="23"/>
-        <v>1.0584261203590295E-4</v>
+        <v>8.303575427643815E-5</v>
       </c>
       <c r="AA7" s="11">
         <f t="shared" si="23"/>
-        <v>1.0349055399066012E-4</v>
+        <v>8.1190515292517505E-5</v>
       </c>
       <c r="AB7" s="11">
         <f t="shared" si="23"/>
-        <v>1.0113849594541816E-4</v>
+        <v>7.9345276308596425E-5</v>
       </c>
       <c r="AC7" s="11">
         <f t="shared" si="23"/>
-        <v>9.8786437900175335E-5</v>
+        <v>7.750003732467578E-5</v>
       </c>
       <c r="AD7" s="11">
         <f t="shared" si="23"/>
-        <v>9.6434379854933375E-5</v>
+        <v>7.5654798340754701E-5</v>
       </c>
       <c r="AE7" s="11">
         <f t="shared" si="23"/>
-        <v>9.4082321809691415E-5</v>
+        <v>7.3809559356834056E-5</v>
       </c>
       <c r="AF7" s="11">
         <f t="shared" si="23"/>
-        <v>9.1730263764448587E-5</v>
+        <v>7.1964320372912977E-5</v>
       </c>
       <c r="AG7" s="11">
         <f t="shared" si="23"/>
-        <v>8.9378205719206627E-5</v>
+        <v>7.0119081388992331E-5</v>
       </c>
       <c r="AH7" s="11">
         <f t="shared" si="23"/>
-        <v>8.7026147673964667E-5</v>
+        <v>6.8273842405071686E-5</v>
       </c>
       <c r="AI7" s="11">
         <f t="shared" si="23"/>
-        <v>8.4674089628721839E-5</v>
+        <v>6.6428603421150607E-5</v>
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">
@@ -5617,7 +5789,7 @@
         <f t="shared" si="24"/>
         <v>8.0429393491877576E-6</v>
       </c>
-      <c r="O8" s="28">
+      <c r="O8" s="11">
         <f t="shared" si="24"/>
         <v>8.0429393491877576E-6</v>
       </c>
@@ -5715,7 +5887,7 @@
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:AI8"/>
+  <dimension ref="A1:AI17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.140625" customWidth="1"/>
@@ -5834,139 +6006,139 @@
       </c>
       <c r="B2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,B$1)</f>
-        <v>1.0662663138431686E-5</v>
+        <v>8.3650833937745032E-6</v>
       </c>
       <c r="C2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,C$1)</f>
-        <v>1.0349055399066077E-5</v>
+        <v>8.1190515292517938E-6</v>
       </c>
       <c r="D2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,D$1)</f>
-        <v>1.0035447659700468E-5</v>
+        <v>7.8730196647289761E-6</v>
       </c>
       <c r="E2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,E$1)</f>
-        <v>9.7218399203347506E-6</v>
+        <v>7.6269878002061583E-6</v>
       </c>
       <c r="F2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,F$1)</f>
-        <v>9.4082321809691415E-6</v>
+        <v>7.3809559356834489E-6</v>
       </c>
       <c r="G2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,G$1)</f>
-        <v>9.0946244416035323E-6</v>
+        <v>7.1349240711606312E-6</v>
       </c>
       <c r="H2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,H$1)</f>
-        <v>8.7810167022379232E-6</v>
+        <v>6.8888922066378134E-6</v>
       </c>
       <c r="I2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,I$1)</f>
-        <v>8.4674089628722056E-6</v>
+        <v>6.642860342115104E-6</v>
       </c>
       <c r="J2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,J$1)</f>
-        <v>8.1538012235065965E-6</v>
+        <v>6.3968284775922863E-6</v>
       </c>
       <c r="K2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,K$1)</f>
-        <v>7.8401934841409874E-6</v>
+        <v>6.1507966130694685E-6</v>
       </c>
       <c r="L2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,L$1)</f>
-        <v>7.5265857447752698E-6</v>
+        <v>5.9047647485467591E-6</v>
       </c>
       <c r="M2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,M$1)</f>
-        <v>7.2129780054096607E-6</v>
+        <v>5.6587328840239414E-6</v>
       </c>
       <c r="N2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,N$1)</f>
-        <v>6.8993702660440515E-6</v>
+        <v>5.4127010195011236E-6</v>
       </c>
       <c r="O2" s="11">
         <f>TREND('DoE Data'!$B$29:$C$29,'DoE Data'!$B$22:$C$22,O$1)</f>
-        <v>6.5857625266784424E-6</v>
+        <v>5.1666691549784143E-6</v>
       </c>
       <c r="P2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,P$1)</f>
-        <v>6.4681596244162848E-6</v>
+        <v>5.074407205782344E-6</v>
       </c>
       <c r="Q2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,Q$1)</f>
-        <v>6.3505567221541542E-6</v>
+        <v>4.9821452565863009E-6</v>
       </c>
       <c r="R2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,R$1)</f>
-        <v>6.2329538198920508E-6</v>
+        <v>4.8898833073902578E-6</v>
       </c>
       <c r="S2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,S$1)</f>
-        <v>6.1153509176299203E-6</v>
+        <v>4.7976213581942147E-6</v>
       </c>
       <c r="T2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,T$1)</f>
-        <v>5.9977480153678168E-6</v>
+        <v>4.7053594089981716E-6</v>
       </c>
       <c r="U2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,U$1)</f>
-        <v>5.8801451131057134E-6</v>
+        <v>4.6130974598021285E-6</v>
       </c>
       <c r="V2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,V$1)</f>
-        <v>5.7625422108435829E-6</v>
+        <v>4.5208355106060854E-6</v>
       </c>
       <c r="W2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,W$1)</f>
-        <v>5.6449393085814795E-6</v>
+        <v>4.4285735614100423E-6</v>
       </c>
       <c r="X2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,X$1)</f>
-        <v>5.527336406319376E-6</v>
+        <v>4.3363116122139991E-6</v>
       </c>
       <c r="Y2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,Y$1)</f>
-        <v>5.4097335040572455E-6</v>
+        <v>4.244049663017956E-6</v>
       </c>
       <c r="Z2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,Z$1)</f>
-        <v>5.2921306017951421E-6</v>
+        <v>4.1517877138219129E-6</v>
       </c>
       <c r="AA2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,AA$1)</f>
-        <v>5.1745276995330115E-6</v>
+        <v>4.0595257646258698E-6</v>
       </c>
       <c r="AB2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,AB$1)</f>
-        <v>5.0569247972709081E-6</v>
+        <v>3.9672638154298267E-6</v>
       </c>
       <c r="AC2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,AC$1)</f>
-        <v>4.9393218950088047E-6</v>
+        <v>3.8750018662337836E-6</v>
       </c>
       <c r="AD2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,AD$1)</f>
-        <v>4.8217189927466742E-6</v>
+        <v>3.7827399170377405E-6</v>
       </c>
       <c r="AE2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,AE$1)</f>
-        <v>4.7041160904845707E-6</v>
+        <v>3.6904779678416974E-6</v>
       </c>
       <c r="AF2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,AF$1)</f>
-        <v>4.5865131882224402E-6</v>
+        <v>3.5982160186456542E-6</v>
       </c>
       <c r="AG2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,AG$1)</f>
-        <v>4.4689102859603368E-6</v>
+        <v>3.5059540694496111E-6</v>
       </c>
       <c r="AH2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,AH$1)</f>
-        <v>4.3513073836982333E-6</v>
+        <v>3.413692120253568E-6</v>
       </c>
       <c r="AI2" s="11">
         <f>TREND('DoE Data'!$C$29:$D$29,'DoE Data'!$C$22:$D$22,AI$1)</f>
-        <v>4.2337044814361028E-6</v>
+        <v>3.3214301710575249E-6</v>
       </c>
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.25">
@@ -6539,139 +6711,139 @@
       </c>
       <c r="B7" s="11">
         <f>B2</f>
-        <v>1.0662663138431686E-5</v>
+        <v>8.3650833937745032E-6</v>
       </c>
       <c r="C7" s="11">
         <f t="shared" ref="C7:AI7" si="2">C2</f>
-        <v>1.0349055399066077E-5</v>
+        <v>8.1190515292517938E-6</v>
       </c>
       <c r="D7" s="11">
         <f t="shared" si="2"/>
-        <v>1.0035447659700468E-5</v>
+        <v>7.8730196647289761E-6</v>
       </c>
       <c r="E7" s="11">
         <f t="shared" si="2"/>
-        <v>9.7218399203347506E-6</v>
+        <v>7.6269878002061583E-6</v>
       </c>
       <c r="F7" s="11">
         <f t="shared" si="2"/>
-        <v>9.4082321809691415E-6</v>
+        <v>7.3809559356834489E-6</v>
       </c>
       <c r="G7" s="11">
         <f t="shared" si="2"/>
-        <v>9.0946244416035323E-6</v>
+        <v>7.1349240711606312E-6</v>
       </c>
       <c r="H7" s="11">
         <f t="shared" si="2"/>
-        <v>8.7810167022379232E-6</v>
+        <v>6.8888922066378134E-6</v>
       </c>
       <c r="I7" s="11">
         <f t="shared" si="2"/>
-        <v>8.4674089628722056E-6</v>
+        <v>6.642860342115104E-6</v>
       </c>
       <c r="J7" s="11">
         <f t="shared" si="2"/>
-        <v>8.1538012235065965E-6</v>
+        <v>6.3968284775922863E-6</v>
       </c>
       <c r="K7" s="11">
         <f t="shared" si="2"/>
-        <v>7.8401934841409874E-6</v>
+        <v>6.1507966130694685E-6</v>
       </c>
       <c r="L7" s="11">
         <f t="shared" si="2"/>
-        <v>7.5265857447752698E-6</v>
+        <v>5.9047647485467591E-6</v>
       </c>
       <c r="M7" s="11">
         <f t="shared" si="2"/>
-        <v>7.2129780054096607E-6</v>
+        <v>5.6587328840239414E-6</v>
       </c>
       <c r="N7" s="11">
         <f t="shared" si="2"/>
-        <v>6.8993702660440515E-6</v>
+        <v>5.4127010195011236E-6</v>
       </c>
       <c r="O7" s="11">
         <f t="shared" si="2"/>
-        <v>6.5857625266784424E-6</v>
+        <v>5.1666691549784143E-6</v>
       </c>
       <c r="P7" s="11">
         <f t="shared" si="2"/>
-        <v>6.4681596244162848E-6</v>
+        <v>5.074407205782344E-6</v>
       </c>
       <c r="Q7" s="11">
         <f t="shared" si="2"/>
-        <v>6.3505567221541542E-6</v>
+        <v>4.9821452565863009E-6</v>
       </c>
       <c r="R7" s="11">
         <f t="shared" si="2"/>
-        <v>6.2329538198920508E-6</v>
+        <v>4.8898833073902578E-6</v>
       </c>
       <c r="S7" s="11">
         <f t="shared" si="2"/>
-        <v>6.1153509176299203E-6</v>
+        <v>4.7976213581942147E-6</v>
       </c>
       <c r="T7" s="11">
         <f t="shared" si="2"/>
-        <v>5.9977480153678168E-6</v>
+        <v>4.7053594089981716E-6</v>
       </c>
       <c r="U7" s="11">
         <f t="shared" si="2"/>
-        <v>5.8801451131057134E-6</v>
+        <v>4.6130974598021285E-6</v>
       </c>
       <c r="V7" s="11">
         <f t="shared" si="2"/>
-        <v>5.7625422108435829E-6</v>
+        <v>4.5208355106060854E-6</v>
       </c>
       <c r="W7" s="11">
         <f t="shared" si="2"/>
-        <v>5.6449393085814795E-6</v>
+        <v>4.4285735614100423E-6</v>
       </c>
       <c r="X7" s="11">
         <f t="shared" si="2"/>
-        <v>5.527336406319376E-6</v>
+        <v>4.3363116122139991E-6</v>
       </c>
       <c r="Y7" s="11">
         <f t="shared" si="2"/>
-        <v>5.4097335040572455E-6</v>
+        <v>4.244049663017956E-6</v>
       </c>
       <c r="Z7" s="11">
         <f t="shared" si="2"/>
-        <v>5.2921306017951421E-6</v>
+        <v>4.1517877138219129E-6</v>
       </c>
       <c r="AA7" s="11">
         <f t="shared" si="2"/>
-        <v>5.1745276995330115E-6</v>
+        <v>4.0595257646258698E-6</v>
       </c>
       <c r="AB7" s="11">
         <f t="shared" si="2"/>
-        <v>5.0569247972709081E-6</v>
+        <v>3.9672638154298267E-6</v>
       </c>
       <c r="AC7" s="11">
         <f t="shared" si="2"/>
-        <v>4.9393218950088047E-6</v>
+        <v>3.8750018662337836E-6</v>
       </c>
       <c r="AD7" s="11">
         <f t="shared" si="2"/>
-        <v>4.8217189927466742E-6</v>
+        <v>3.7827399170377405E-6</v>
       </c>
       <c r="AE7" s="11">
         <f t="shared" si="2"/>
-        <v>4.7041160904845707E-6</v>
+        <v>3.6904779678416974E-6</v>
       </c>
       <c r="AF7" s="11">
         <f t="shared" si="2"/>
-        <v>4.5865131882224402E-6</v>
+        <v>3.5982160186456542E-6</v>
       </c>
       <c r="AG7" s="11">
         <f t="shared" si="2"/>
-        <v>4.4689102859603368E-6</v>
+        <v>3.5059540694496111E-6</v>
       </c>
       <c r="AH7" s="11">
         <f t="shared" si="2"/>
-        <v>4.3513073836982333E-6</v>
+        <v>3.413692120253568E-6</v>
       </c>
       <c r="AI7" s="11">
         <f t="shared" si="2"/>
-        <v>4.2337044814361028E-6</v>
+        <v>3.3214301710575249E-6</v>
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">
@@ -6814,6 +6986,30 @@
         <f t="shared" si="3"/>
         <v>3.7801814941182461E-7</v>
       </c>
+    </row>
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="B10" s="11"/>
+    </row>
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="B11" s="11"/>
+    </row>
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="B12" s="11"/>
+    </row>
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="B13" s="11"/>
+    </row>
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="B14" s="11"/>
+    </row>
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="B15" s="11"/>
+    </row>
+    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="B16" s="11"/>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6944,59 +7140,59 @@
       </c>
       <c r="B2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,B$1)</f>
-        <v>1.6130528470100847E-5</v>
+        <v>1.6130528470100955E-5</v>
       </c>
       <c r="C2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,C$1)</f>
-        <v>1.5656477990836542E-5</v>
+        <v>1.565647799083665E-5</v>
       </c>
       <c r="D2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,D$1)</f>
-        <v>1.5182427511572236E-5</v>
+        <v>1.5182427511572453E-5</v>
       </c>
       <c r="E2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,E$1)</f>
-        <v>1.4708377032307931E-5</v>
+        <v>1.4708377032308147E-5</v>
       </c>
       <c r="F2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,F$1)</f>
-        <v>1.4234326553043733E-5</v>
+        <v>1.4234326553043842E-5</v>
       </c>
       <c r="G2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,G$1)</f>
-        <v>1.3760276073779428E-5</v>
+        <v>1.3760276073779536E-5</v>
       </c>
       <c r="H2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,H$1)</f>
-        <v>1.3286225594515122E-5</v>
+        <v>1.3286225594515231E-5</v>
       </c>
       <c r="I2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,I$1)</f>
-        <v>1.2812175115250817E-5</v>
+        <v>1.2812175115250925E-5</v>
       </c>
       <c r="J2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,J$1)</f>
-        <v>1.2338124635986512E-5</v>
+        <v>1.233812463598662E-5</v>
       </c>
       <c r="K2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,K$1)</f>
-        <v>1.1864074156722314E-5</v>
+        <v>1.1864074156722423E-5</v>
       </c>
       <c r="L2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,L$1)</f>
-        <v>1.1390023677458009E-5</v>
+        <v>1.1390023677458117E-5</v>
       </c>
       <c r="M2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,M$1)</f>
-        <v>1.0915973198193703E-5</v>
+        <v>1.0915973198193812E-5</v>
       </c>
       <c r="N2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,N$1)</f>
-        <v>1.0441922718929398E-5</v>
+        <v>1.0441922718929506E-5</v>
       </c>
       <c r="O2" s="11">
         <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,O$1)</f>
-        <v>9.9678722396650925E-6</v>
+        <v>9.9678722396652009E-6</v>
       </c>
       <c r="P2" s="13">
         <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,P$1)</f>
@@ -7649,59 +7845,59 @@
       </c>
       <c r="B7" s="11">
         <f>B2</f>
-        <v>1.6130528470100847E-5</v>
+        <v>1.6130528470100955E-5</v>
       </c>
       <c r="C7" s="11">
         <f t="shared" ref="C7:AI8" si="2">C2</f>
-        <v>1.5656477990836542E-5</v>
+        <v>1.565647799083665E-5</v>
       </c>
       <c r="D7" s="11">
         <f t="shared" si="2"/>
-        <v>1.5182427511572236E-5</v>
+        <v>1.5182427511572453E-5</v>
       </c>
       <c r="E7" s="11">
         <f t="shared" si="2"/>
-        <v>1.4708377032307931E-5</v>
+        <v>1.4708377032308147E-5</v>
       </c>
       <c r="F7" s="11">
         <f t="shared" si="2"/>
-        <v>1.4234326553043733E-5</v>
+        <v>1.4234326553043842E-5</v>
       </c>
       <c r="G7" s="11">
         <f t="shared" si="2"/>
-        <v>1.3760276073779428E-5</v>
+        <v>1.3760276073779536E-5</v>
       </c>
       <c r="H7" s="11">
         <f t="shared" si="2"/>
-        <v>1.3286225594515122E-5</v>
+        <v>1.3286225594515231E-5</v>
       </c>
       <c r="I7" s="11">
         <f t="shared" si="2"/>
-        <v>1.2812175115250817E-5</v>
+        <v>1.2812175115250925E-5</v>
       </c>
       <c r="J7" s="11">
         <f t="shared" si="2"/>
-        <v>1.2338124635986512E-5</v>
+        <v>1.233812463598662E-5</v>
       </c>
       <c r="K7" s="11">
         <f t="shared" si="2"/>
-        <v>1.1864074156722314E-5</v>
+        <v>1.1864074156722423E-5</v>
       </c>
       <c r="L7" s="11">
         <f t="shared" si="2"/>
-        <v>1.1390023677458009E-5</v>
+        <v>1.1390023677458117E-5</v>
       </c>
       <c r="M7" s="11">
         <f t="shared" si="2"/>
-        <v>1.0915973198193703E-5</v>
+        <v>1.0915973198193812E-5</v>
       </c>
       <c r="N7" s="11">
         <f t="shared" si="2"/>
-        <v>1.0441922718929398E-5</v>
+        <v>1.0441922718929506E-5</v>
       </c>
       <c r="O7" s="11">
         <f t="shared" si="2"/>
-        <v>9.9678722396650925E-6</v>
+        <v>9.9678722396652009E-6</v>
       </c>
       <c r="P7" s="11">
         <f t="shared" si="2"/>

</xml_diff>

<commit_message>
Adds hydrogen production equipment capital cost R&D lever (#386)
</commit_message>
<xml_diff>
--- a/InputData/hydgn/HPEC/Hydrogen Production Eqpt Costs.xlsx
+++ b/InputData/hydgn/HPEC/Hydrogen Production Eqpt Costs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\hydgn\HPEC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\hydgn\HPEC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{367FBC82-7E96-48E1-B217-997B48B264DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{226829CA-22C7-4710-951B-DA08E09623C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2880" yWindow="2505" windowWidth="21600" windowHeight="14655" tabRatio="658" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26490" yWindow="1290" windowWidth="26130" windowHeight="14580" tabRatio="658" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -20,8 +20,6 @@
     <sheet name="Conversion Factors" sheetId="4" r:id="rId5"/>
     <sheet name="HPEC" sheetId="3" r:id="rId6"/>
     <sheet name="HPEO" sheetId="5" r:id="rId7"/>
-    <sheet name="LHPEC" sheetId="8" r:id="rId8"/>
-    <sheet name="LHPEO" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="btu_per_kwh">'Conversion Factors'!$A$3</definedName>
@@ -49,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="203">
   <si>
     <t>HPEC Hydrogen Production Equipment CapEx</t>
   </si>
@@ -561,12 +559,6 @@
   </si>
   <si>
     <t>other</t>
-  </si>
-  <si>
-    <t>Levelized CapEx Cost ($/BTU)</t>
-  </si>
-  <si>
-    <t>Levelized OpEx Cost ($/BTU)</t>
   </si>
   <si>
     <t>kg H2/yr</t>
@@ -2084,11 +2076,11 @@
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="11">
         <f>B32/B21</f>
-        <v>4.7252268676478081E-7</v>
+        <v>1.7132403345724911E-6</v>
       </c>
       <c r="B32" s="19">
         <f>HPEO!B3*B21*(1+B28)</f>
-        <v>8.68346787400779E-2</v>
+        <v>0.31483921983877583</v>
       </c>
       <c r="C32" t="s">
         <v>93</v>
@@ -2097,7 +2089,7 @@
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="11">
         <f>SUM(A30:A32)</f>
-        <v>1.5123984873249478E-5</v>
+        <v>1.6364702521057188E-5</v>
       </c>
     </row>
   </sheetData>
@@ -2145,7 +2137,7 @@
         <v>137</v>
       </c>
       <c r="C5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D5">
         <f>500000*365</f>
@@ -2297,7 +2289,7 @@
         <v>0.18434466000000002</v>
       </c>
       <c r="C35" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.25">
@@ -2306,20 +2298,20 @@
         <v>1.3705922676579926E-6</v>
       </c>
       <c r="C36" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C39" t="s">
         <v>135</v>
@@ -2328,314 +2320,314 @@
         <v>136</v>
       </c>
       <c r="E39" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="G39">
         <v>216000000</v>
       </c>
       <c r="H39" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G40">
         <f>G39/D5</f>
         <v>1.1835616438356165</v>
       </c>
       <c r="H40" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C41" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D41">
         <v>500</v>
       </c>
       <c r="E41" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G41" s="11">
         <f>G40/'IEA Data'!B18*'IEA Data'!B19*About!A75</f>
         <v>8.0429393491877576E-6</v>
       </c>
       <c r="H41" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C42" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D42">
         <v>25</v>
       </c>
       <c r="E42" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C43" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D43">
         <v>2.7</v>
       </c>
       <c r="E43" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C44" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D44" s="25">
         <v>1800</v>
       </c>
       <c r="E44" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C45" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D45">
         <v>24.8</v>
       </c>
       <c r="E45" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C46" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D46">
         <v>0.75</v>
       </c>
       <c r="E46" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C48" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D48">
         <v>700</v>
       </c>
       <c r="E48" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C49" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D49">
         <v>24</v>
       </c>
       <c r="E49" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C50" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D50">
         <v>3</v>
       </c>
       <c r="E50" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C51" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D51" s="25">
         <v>1246</v>
       </c>
       <c r="E51" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C52" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D52">
         <v>34.299999999999997</v>
       </c>
       <c r="E52" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C53" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D53">
         <v>0.75</v>
       </c>
       <c r="E53" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C56" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D56">
         <v>320</v>
       </c>
       <c r="E56" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C57" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D57">
         <v>23</v>
       </c>
       <c r="E57" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C59" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D59">
         <v>190</v>
       </c>
       <c r="E59" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C60" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D60">
         <v>22.5</v>
       </c>
       <c r="E60" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="62" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C62" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D62">
         <v>25</v>
       </c>
       <c r="E62" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="63" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C63" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D63">
         <v>23</v>
       </c>
       <c r="E63" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="64" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C64" t="s">
         <v>11</v>
@@ -2644,12 +2636,12 @@
         <v>90</v>
       </c>
       <c r="E64" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C65" t="s">
         <v>11</v>
@@ -2658,49 +2650,49 @@
         <v>99.99</v>
       </c>
       <c r="E65" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C66" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D66" s="25">
         <v>17069</v>
       </c>
       <c r="E66" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C67" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D67">
         <v>35.299999999999997</v>
       </c>
       <c r="E67" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C68" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D68">
         <v>0.6</v>
       </c>
       <c r="E68" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -2774,7 +2766,7 @@
         <v>82</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
@@ -2791,7 +2783,7 @@
         <v>207843137.25490195</v>
       </c>
       <c r="E24" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
@@ -2808,7 +2800,7 @@
         <v>11.38866505506312</v>
       </c>
       <c r="E25" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
@@ -2825,7 +2817,7 @@
         <v>6.6428603421150552E-5</v>
       </c>
       <c r="E26" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
@@ -2842,10 +2834,10 @@
         <v>10392156.862745099</v>
       </c>
       <c r="E27" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
@@ -2862,7 +2854,7 @@
         <v>0.56943325275315615</v>
       </c>
       <c r="E28" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
@@ -2879,7 +2871,7 @@
         <v>3.3214301710575287E-6</v>
       </c>
       <c r="E29" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
@@ -3911,7 +3903,7 @@
     </row>
     <row r="61" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B61" s="14">
         <f>SUM(B56:B59)/(1+$B$46)^(B52-1)</f>
@@ -4036,7 +4028,7 @@
     </row>
     <row r="62" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B62" s="14">
         <f>(B57+B59)/(1+$B$46)^(B52-1)</f>
@@ -4161,7 +4153,7 @@
     </row>
     <row r="63" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B63">
         <f>B58/(1+$B$46)^(B52-1)</f>
@@ -4429,7 +4421,7 @@
         <v>119</v>
       </c>
       <c r="E67" s="23" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G67">
         <f>SUM(B63:J63)/SUM(B64:J64)</f>
@@ -4442,10 +4434,10 @@
         <v>1.1388665055063121</v>
       </c>
       <c r="C68" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E68" s="23" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H68">
         <f>SUM(B64:AE64)</f>
@@ -4519,7 +4511,7 @@
     </row>
     <row r="76" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B76" s="15" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="77" spans="2:38" x14ac:dyDescent="0.25">
@@ -5890,7 +5882,7 @@
   <dimension ref="A1:AI17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.140625" customWidth="1"/>
+    <col min="1" max="1" width="41.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
@@ -6146,140 +6138,140 @@
         <v>16</v>
       </c>
       <c r="B3" s="11">
-        <f>HPEC!B3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="C3" s="11">
-        <f>HPEC!C3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="D3" s="11">
-        <f>HPEC!D3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="E3" s="11">
-        <f>HPEC!E3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="F3" s="11">
-        <f>HPEC!F3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="G3" s="11">
-        <f>HPEC!G3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="H3" s="11">
-        <f>HPEC!H3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="I3" s="11">
-        <f>HPEC!I3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="J3" s="11">
-        <f>HPEC!J3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="K3" s="11">
-        <f>HPEC!K3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="L3" s="11">
-        <f>HPEC!L3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="M3" s="11">
-        <f>HPEC!M3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="N3" s="11">
-        <f>HPEC!N3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="O3" s="11">
-        <f>HPEC!O3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="P3" s="11">
-        <f>HPEC!P3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="Q3" s="11">
-        <f>HPEC!Q3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="R3" s="11">
-        <f>HPEC!R3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="S3" s="11">
-        <f>HPEC!S3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="T3" s="11">
-        <f>HPEC!T3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="U3" s="11">
-        <f>HPEC!U3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="V3" s="11">
-        <f>HPEC!V3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="W3" s="11">
-        <f>HPEC!W3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="X3" s="11">
-        <f>HPEC!X3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="Y3" s="11">
-        <f>HPEC!Y3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="Z3" s="11">
-        <f>HPEC!Z3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AA3" s="11">
-        <f>HPEC!AA3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AB3" s="11">
-        <f>HPEC!AB3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AC3" s="11">
-        <f>HPEC!AC3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AD3" s="11">
-        <f>HPEC!AD3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AE3" s="11">
-        <f>HPEC!AE3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AF3" s="11">
-        <f>HPEC!AF3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AG3" s="11">
-        <f>HPEC!AG3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AH3" s="11">
-        <f>HPEC!AH3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AI3" s="11">
-        <f>HPEC!AI3*'IEA Data'!$D$8</f>
-        <v>3.7801814941182461E-7</v>
+        <f>'Reformer data'!$B$36</f>
+        <v>1.3705922676579926E-6</v>
       </c>
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.25">
@@ -6287,140 +6279,140 @@
         <v>19</v>
       </c>
       <c r="B4" s="11">
-        <f>HPEC!B4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>B3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="C4" s="11">
-        <f>HPEC!C4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>C3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="D4" s="11">
-        <f>HPEC!D4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>D3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="E4" s="11">
-        <f>HPEC!E4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>E3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="F4" s="11">
-        <f>HPEC!F4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>F3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="G4" s="11">
-        <f>HPEC!G4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>G3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="H4" s="11">
-        <f>HPEC!H4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>H3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="I4" s="11">
-        <f>HPEC!I4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>I3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="J4" s="11">
-        <f>HPEC!J4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>J3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="K4" s="11">
-        <f>HPEC!K4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>K3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="L4" s="11">
-        <f>HPEC!L4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>L3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="M4" s="11">
-        <f>HPEC!M4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>M3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="N4" s="11">
-        <f>HPEC!N4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>N3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="O4" s="11">
-        <f>HPEC!O4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>O3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="P4" s="11">
-        <f>HPEC!P4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>P3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="Q4" s="11">
-        <f>HPEC!Q4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>Q3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="R4" s="11">
-        <f>HPEC!R4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>R3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="S4" s="11">
-        <f>HPEC!S4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>S3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="T4" s="11">
-        <f>HPEC!T4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>T3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="U4" s="11">
-        <f>HPEC!U4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>U3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="V4" s="11">
-        <f>HPEC!V4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>V3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="W4" s="11">
-        <f>HPEC!W4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>W3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="X4" s="11">
-        <f>HPEC!X4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>X3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="Y4" s="11">
-        <f>HPEC!Y4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>Y3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="Z4" s="11">
-        <f>HPEC!Z4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>Z3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AA4" s="11">
-        <f>HPEC!AA4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>AA3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AB4" s="11">
-        <f>HPEC!AB4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>AB3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AC4" s="11">
-        <f>HPEC!AC4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>AC3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AD4" s="11">
-        <f>HPEC!AD4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>AD3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AE4" s="11">
-        <f>HPEC!AE4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>AE3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AF4" s="11">
-        <f>HPEC!AF4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>AF3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AG4" s="11">
-        <f>HPEC!AG4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>AG3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AH4" s="11">
-        <f>HPEC!AH4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>AH3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AI4" s="11">
-        <f>HPEC!AI4*'IEA Data'!$D$12</f>
-        <v>1.1799257177105119E-6</v>
+        <f>AI3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
+        <v>4.021408082029495E-6</v>
       </c>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.25">
@@ -6429,139 +6421,139 @@
       </c>
       <c r="B5" s="11">
         <f>B4</f>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="C5" s="11">
         <f t="shared" ref="C5:AI5" si="0">C4</f>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="D5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="E5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="F5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="G5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="H5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="I5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="J5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="K5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="L5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="M5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="N5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="O5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="P5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="Q5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="R5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="S5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="T5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="U5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="V5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="W5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="X5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="Y5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="Z5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AA5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AB5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AC5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AD5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AE5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AF5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AG5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AH5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
       <c r="AI5" s="11">
         <f t="shared" si="0"/>
-        <v>1.1799257177105119E-6</v>
+        <v>4.021408082029495E-6</v>
       </c>
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.25">
@@ -6569,140 +6561,140 @@
         <v>65</v>
       </c>
       <c r="B6" s="11">
-        <f>B3*0.95</f>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="C6">
-        <f t="shared" ref="C6:AI6" si="1">$B6</f>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="D6">
+        <f>B3*0.85</f>
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="C6" s="11">
+        <f t="shared" ref="C6:AI6" si="1">C3*0.85</f>
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="D6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="E6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="E6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="F6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="F6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="G6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="G6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="H6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="H6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="I6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="I6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="J6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="J6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="K6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="K6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="L6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="L6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="M6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="M6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="N6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="N6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="O6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="O6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="P6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="P6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="Q6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="Q6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="R6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="R6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="S6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="S6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="T6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="T6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="U6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="U6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="V6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="V6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="W6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="W6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="X6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="X6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="Y6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="Y6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="Z6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="Z6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="AA6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="AA6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="AB6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="AB6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="AC6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="AC6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="AD6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="AD6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="AE6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="AE6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="AF6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="AF6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="AG6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="AG6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="AH6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="AH6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
-      </c>
-      <c r="AI6">
+        <v>1.1650034275092937E-6</v>
+      </c>
+      <c r="AI6" s="11">
         <f t="shared" si="1"/>
-        <v>3.5911724194123339E-7</v>
+        <v>1.1650034275092937E-6</v>
       </c>
     </row>
     <row r="7" spans="1:35" x14ac:dyDescent="0.25">
@@ -6852,139 +6844,139 @@
       </c>
       <c r="B8" s="11">
         <f>B3</f>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="C8" s="11">
         <f t="shared" ref="C8:AI8" si="3">C3</f>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="D8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="E8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="F8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="G8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="H8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="I8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="J8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="K8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="L8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="M8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="N8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="O8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="P8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="Q8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="R8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="S8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="T8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="U8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="V8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="W8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="X8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="Y8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="Z8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AA8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AB8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AC8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AD8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AE8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AF8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AG8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AH8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
       <c r="AI8" s="11">
         <f t="shared" si="3"/>
-        <v>3.7801814941182461E-7</v>
+        <v>1.3705922676579926E-6</v>
       </c>
     </row>
     <row r="10" spans="1:35" x14ac:dyDescent="0.25">
@@ -7010,2226 +7002,6 @@
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="11"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CCAC499-E3B9-41CD-9477-496757FA6389}">
-  <sheetPr>
-    <tabColor theme="8" tint="-0.249977111117893"/>
-  </sheetPr>
-  <dimension ref="A1:AI8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="41.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="B1" s="9">
-        <v>2017</v>
-      </c>
-      <c r="C1">
-        <v>2018</v>
-      </c>
-      <c r="D1" s="9">
-        <v>2019</v>
-      </c>
-      <c r="E1">
-        <v>2020</v>
-      </c>
-      <c r="F1" s="9">
-        <v>2021</v>
-      </c>
-      <c r="G1">
-        <v>2022</v>
-      </c>
-      <c r="H1" s="9">
-        <v>2023</v>
-      </c>
-      <c r="I1">
-        <v>2024</v>
-      </c>
-      <c r="J1" s="9">
-        <v>2025</v>
-      </c>
-      <c r="K1">
-        <v>2026</v>
-      </c>
-      <c r="L1" s="9">
-        <v>2027</v>
-      </c>
-      <c r="M1">
-        <v>2028</v>
-      </c>
-      <c r="N1" s="9">
-        <v>2029</v>
-      </c>
-      <c r="O1" s="12">
-        <v>2030</v>
-      </c>
-      <c r="P1" s="10">
-        <v>2031</v>
-      </c>
-      <c r="Q1">
-        <v>2032</v>
-      </c>
-      <c r="R1" s="9">
-        <v>2033</v>
-      </c>
-      <c r="S1">
-        <v>2034</v>
-      </c>
-      <c r="T1" s="9">
-        <v>2035</v>
-      </c>
-      <c r="U1">
-        <v>2036</v>
-      </c>
-      <c r="V1" s="9">
-        <v>2037</v>
-      </c>
-      <c r="W1">
-        <v>2038</v>
-      </c>
-      <c r="X1" s="9">
-        <v>2039</v>
-      </c>
-      <c r="Y1">
-        <v>2040</v>
-      </c>
-      <c r="Z1" s="9">
-        <v>2041</v>
-      </c>
-      <c r="AA1">
-        <v>2042</v>
-      </c>
-      <c r="AB1" s="9">
-        <v>2043</v>
-      </c>
-      <c r="AC1">
-        <v>2044</v>
-      </c>
-      <c r="AD1" s="9">
-        <v>2045</v>
-      </c>
-      <c r="AE1">
-        <v>2046</v>
-      </c>
-      <c r="AF1" s="9">
-        <v>2047</v>
-      </c>
-      <c r="AG1">
-        <v>2048</v>
-      </c>
-      <c r="AH1" s="9">
-        <v>2049</v>
-      </c>
-      <c r="AI1">
-        <v>2050</v>
-      </c>
-    </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,B$1)</f>
-        <v>1.6130528470100955E-5</v>
-      </c>
-      <c r="C2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,C$1)</f>
-        <v>1.565647799083665E-5</v>
-      </c>
-      <c r="D2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,D$1)</f>
-        <v>1.5182427511572453E-5</v>
-      </c>
-      <c r="E2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,E$1)</f>
-        <v>1.4708377032308147E-5</v>
-      </c>
-      <c r="F2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,F$1)</f>
-        <v>1.4234326553043842E-5</v>
-      </c>
-      <c r="G2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,G$1)</f>
-        <v>1.3760276073779536E-5</v>
-      </c>
-      <c r="H2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,H$1)</f>
-        <v>1.3286225594515231E-5</v>
-      </c>
-      <c r="I2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,I$1)</f>
-        <v>1.2812175115250925E-5</v>
-      </c>
-      <c r="J2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,J$1)</f>
-        <v>1.233812463598662E-5</v>
-      </c>
-      <c r="K2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,K$1)</f>
-        <v>1.1864074156722423E-5</v>
-      </c>
-      <c r="L2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,L$1)</f>
-        <v>1.1390023677458117E-5</v>
-      </c>
-      <c r="M2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,M$1)</f>
-        <v>1.0915973198193812E-5</v>
-      </c>
-      <c r="N2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,N$1)</f>
-        <v>1.0441922718929506E-5</v>
-      </c>
-      <c r="O2" s="11">
-        <f>TREND('DoE Data'!$B$74:$C$74,'DoE Data'!$B$22:$C$22,O$1)</f>
-        <v>9.9678722396652009E-6</v>
-      </c>
-      <c r="P2" s="13">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,P$1)</f>
-        <v>9.7897830055632303E-6</v>
-      </c>
-      <c r="Q2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,Q$1)</f>
-        <v>9.6116937714612596E-6</v>
-      </c>
-      <c r="R2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,R$1)</f>
-        <v>9.433604537359289E-6</v>
-      </c>
-      <c r="S2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,S$1)</f>
-        <v>9.2555153032572641E-6</v>
-      </c>
-      <c r="T2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,T$1)</f>
-        <v>9.0774260691552935E-6</v>
-      </c>
-      <c r="U2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,U$1)</f>
-        <v>8.8993368350533228E-6</v>
-      </c>
-      <c r="V2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,V$1)</f>
-        <v>8.721247600951298E-6</v>
-      </c>
-      <c r="W2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,W$1)</f>
-        <v>8.5431583668493273E-6</v>
-      </c>
-      <c r="X2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,X$1)</f>
-        <v>8.3650691327473567E-6</v>
-      </c>
-      <c r="Y2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,Y$1)</f>
-        <v>8.1869798986453318E-6</v>
-      </c>
-      <c r="Z2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,Z$1)</f>
-        <v>8.0088906645433612E-6</v>
-      </c>
-      <c r="AA2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,AA$1)</f>
-        <v>7.8308014304413905E-6</v>
-      </c>
-      <c r="AB2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,AB$1)</f>
-        <v>7.6527121963394199E-6</v>
-      </c>
-      <c r="AC2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,AC$1)</f>
-        <v>7.474622962237395E-6</v>
-      </c>
-      <c r="AD2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,AD$1)</f>
-        <v>7.2965337281354244E-6</v>
-      </c>
-      <c r="AE2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,AE$1)</f>
-        <v>7.1184444940334537E-6</v>
-      </c>
-      <c r="AF2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,AF$1)</f>
-        <v>6.9403552599314289E-6</v>
-      </c>
-      <c r="AG2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,AG$1)</f>
-        <v>6.7622660258294582E-6</v>
-      </c>
-      <c r="AH2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,AH$1)</f>
-        <v>6.5841767917274876E-6</v>
-      </c>
-      <c r="AI2" s="11">
-        <f>TREND('DoE Data'!$C$74:$D$74,'DoE Data'!$C$22:$D$22,AI$1)</f>
-        <v>6.4060875576254627E-6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="C3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="D3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="E3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="F3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="G3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="H3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="I3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="J3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="K3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="L3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="M3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="N3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="O3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="P3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="Q3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="R3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="S3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="T3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="U3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="V3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="W3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="X3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="Y3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="Z3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AA3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AB3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AC3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AD3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AE3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AF3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AG3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AH3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AI3" s="11">
-        <f>'Reformer data'!$G$10</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="11">
-        <f>B3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="C4" s="11">
-        <f>C3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="D4" s="11">
-        <f>D3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="E4" s="11">
-        <f>E3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="F4" s="11">
-        <f>F3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="G4" s="11">
-        <f>G3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="H4" s="11">
-        <f>H3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="I4" s="11">
-        <f>I3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="J4" s="11">
-        <f>J3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="K4" s="11">
-        <f>K3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="L4" s="11">
-        <f>L3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="M4" s="11">
-        <f>M3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="N4" s="11">
-        <f>N3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="O4" s="11">
-        <f>O3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="P4" s="11">
-        <f>P3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="Q4" s="11">
-        <f>Q3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="R4" s="11">
-        <f>R3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="S4" s="11">
-        <f>S3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="T4" s="11">
-        <f>T3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="U4" s="11">
-        <f>U3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="V4" s="11">
-        <f>V3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="W4" s="11">
-        <f>W3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="X4" s="11">
-        <f>X3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="Y4" s="11">
-        <f>Y3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="Z4" s="11">
-        <f>Z3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AA4" s="11">
-        <f>AA3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AB4" s="11">
-        <f>AB3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AC4" s="11">
-        <f>AC3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AD4" s="11">
-        <f>AD3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AE4" s="11">
-        <f>AE3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AF4" s="11">
-        <f>AF3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AG4" s="11">
-        <f>AG3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AH4" s="11">
-        <f>AH3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AI4" s="11">
-        <f>AI3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="11">
-        <f>B4</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="C5" s="11">
-        <f t="shared" ref="C5:AI5" si="0">C4</f>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="D5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="E5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="F5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="G5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="H5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="I5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="J5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="K5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="L5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="M5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="N5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="O5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="P5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="Q5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="R5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="S5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="T5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="U5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="V5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="W5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="X5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="Y5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="Z5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AA5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AB5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AC5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AD5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AE5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AF5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AG5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AH5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-      <c r="AI5" s="11">
-        <f t="shared" si="0"/>
-        <v>2.9907839372523382E-6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="11">
-        <f>B3*0.85</f>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="C6">
-        <f t="shared" ref="C6:AI6" si="1">$B6</f>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="D6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="E6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="F6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="G6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="H6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="I6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="J6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="K6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="L6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="M6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="N6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="O6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="P6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="Q6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="R6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="S6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="T6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="U6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="V6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="W6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="X6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="Y6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="Z6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="AA6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="AB6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="AC6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="AD6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="AE6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="AF6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="AG6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="AH6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-      <c r="AI6">
-        <f t="shared" si="1"/>
-        <v>8.6643122676579916E-7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B7" s="11">
-        <f>B2</f>
-        <v>1.6130528470100955E-5</v>
-      </c>
-      <c r="C7" s="11">
-        <f t="shared" ref="C7:AI8" si="2">C2</f>
-        <v>1.565647799083665E-5</v>
-      </c>
-      <c r="D7" s="11">
-        <f t="shared" si="2"/>
-        <v>1.5182427511572453E-5</v>
-      </c>
-      <c r="E7" s="11">
-        <f t="shared" si="2"/>
-        <v>1.4708377032308147E-5</v>
-      </c>
-      <c r="F7" s="11">
-        <f t="shared" si="2"/>
-        <v>1.4234326553043842E-5</v>
-      </c>
-      <c r="G7" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3760276073779536E-5</v>
-      </c>
-      <c r="H7" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3286225594515231E-5</v>
-      </c>
-      <c r="I7" s="11">
-        <f t="shared" si="2"/>
-        <v>1.2812175115250925E-5</v>
-      </c>
-      <c r="J7" s="11">
-        <f t="shared" si="2"/>
-        <v>1.233812463598662E-5</v>
-      </c>
-      <c r="K7" s="11">
-        <f t="shared" si="2"/>
-        <v>1.1864074156722423E-5</v>
-      </c>
-      <c r="L7" s="11">
-        <f t="shared" si="2"/>
-        <v>1.1390023677458117E-5</v>
-      </c>
-      <c r="M7" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0915973198193812E-5</v>
-      </c>
-      <c r="N7" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0441922718929506E-5</v>
-      </c>
-      <c r="O7" s="11">
-        <f t="shared" si="2"/>
-        <v>9.9678722396652009E-6</v>
-      </c>
-      <c r="P7" s="11">
-        <f t="shared" si="2"/>
-        <v>9.7897830055632303E-6</v>
-      </c>
-      <c r="Q7" s="11">
-        <f t="shared" si="2"/>
-        <v>9.6116937714612596E-6</v>
-      </c>
-      <c r="R7" s="11">
-        <f t="shared" si="2"/>
-        <v>9.433604537359289E-6</v>
-      </c>
-      <c r="S7" s="11">
-        <f t="shared" si="2"/>
-        <v>9.2555153032572641E-6</v>
-      </c>
-      <c r="T7" s="11">
-        <f t="shared" si="2"/>
-        <v>9.0774260691552935E-6</v>
-      </c>
-      <c r="U7" s="11">
-        <f t="shared" si="2"/>
-        <v>8.8993368350533228E-6</v>
-      </c>
-      <c r="V7" s="11">
-        <f t="shared" si="2"/>
-        <v>8.721247600951298E-6</v>
-      </c>
-      <c r="W7" s="11">
-        <f t="shared" si="2"/>
-        <v>8.5431583668493273E-6</v>
-      </c>
-      <c r="X7" s="11">
-        <f t="shared" si="2"/>
-        <v>8.3650691327473567E-6</v>
-      </c>
-      <c r="Y7" s="11">
-        <f t="shared" si="2"/>
-        <v>8.1869798986453318E-6</v>
-      </c>
-      <c r="Z7" s="11">
-        <f t="shared" si="2"/>
-        <v>8.0088906645433612E-6</v>
-      </c>
-      <c r="AA7" s="11">
-        <f t="shared" si="2"/>
-        <v>7.8308014304413905E-6</v>
-      </c>
-      <c r="AB7" s="11">
-        <f t="shared" si="2"/>
-        <v>7.6527121963394199E-6</v>
-      </c>
-      <c r="AC7" s="11">
-        <f t="shared" si="2"/>
-        <v>7.474622962237395E-6</v>
-      </c>
-      <c r="AD7" s="11">
-        <f t="shared" si="2"/>
-        <v>7.2965337281354244E-6</v>
-      </c>
-      <c r="AE7" s="11">
-        <f t="shared" si="2"/>
-        <v>7.1184444940334537E-6</v>
-      </c>
-      <c r="AF7" s="11">
-        <f t="shared" si="2"/>
-        <v>6.9403552599314289E-6</v>
-      </c>
-      <c r="AG7" s="11">
-        <f t="shared" si="2"/>
-        <v>6.7622660258294582E-6</v>
-      </c>
-      <c r="AH7" s="11">
-        <f t="shared" si="2"/>
-        <v>6.5841767917274876E-6</v>
-      </c>
-      <c r="AI7" s="11">
-        <f t="shared" si="2"/>
-        <v>6.4060875576254627E-6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B8" s="11">
-        <f>B3</f>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="C8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="D8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="E8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="F8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="G8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="H8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="I8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="J8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="K8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="L8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="M8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="N8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="O8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="P8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="Q8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="R8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="S8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="T8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="U8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="V8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="W8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="X8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="Y8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="Z8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AA8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AB8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AC8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AD8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AE8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AF8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AG8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AH8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-      <c r="AI8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.0193308550185872E-6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F6400E6-6C48-4F0B-9F72-909A60878C43}">
-  <sheetPr>
-    <tabColor theme="8" tint="-0.249977111117893"/>
-  </sheetPr>
-  <dimension ref="A1:AI8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="41.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="B1" s="9">
-        <v>2017</v>
-      </c>
-      <c r="C1">
-        <v>2018</v>
-      </c>
-      <c r="D1" s="9">
-        <v>2019</v>
-      </c>
-      <c r="E1">
-        <v>2020</v>
-      </c>
-      <c r="F1" s="9">
-        <v>2021</v>
-      </c>
-      <c r="G1">
-        <v>2022</v>
-      </c>
-      <c r="H1" s="9">
-        <v>2023</v>
-      </c>
-      <c r="I1">
-        <v>2024</v>
-      </c>
-      <c r="J1" s="9">
-        <v>2025</v>
-      </c>
-      <c r="K1">
-        <v>2026</v>
-      </c>
-      <c r="L1" s="9">
-        <v>2027</v>
-      </c>
-      <c r="M1">
-        <v>2028</v>
-      </c>
-      <c r="N1" s="9">
-        <v>2029</v>
-      </c>
-      <c r="O1" s="12">
-        <v>2030</v>
-      </c>
-      <c r="P1" s="10">
-        <v>2031</v>
-      </c>
-      <c r="Q1">
-        <v>2032</v>
-      </c>
-      <c r="R1" s="9">
-        <v>2033</v>
-      </c>
-      <c r="S1">
-        <v>2034</v>
-      </c>
-      <c r="T1" s="9">
-        <v>2035</v>
-      </c>
-      <c r="U1">
-        <v>2036</v>
-      </c>
-      <c r="V1" s="9">
-        <v>2037</v>
-      </c>
-      <c r="W1">
-        <v>2038</v>
-      </c>
-      <c r="X1" s="9">
-        <v>2039</v>
-      </c>
-      <c r="Y1">
-        <v>2040</v>
-      </c>
-      <c r="Z1" s="9">
-        <v>2041</v>
-      </c>
-      <c r="AA1">
-        <v>2042</v>
-      </c>
-      <c r="AB1" s="9">
-        <v>2043</v>
-      </c>
-      <c r="AC1">
-        <v>2044</v>
-      </c>
-      <c r="AD1" s="9">
-        <v>2045</v>
-      </c>
-      <c r="AE1">
-        <v>2046</v>
-      </c>
-      <c r="AF1" s="9">
-        <v>2047</v>
-      </c>
-      <c r="AG1">
-        <v>2048</v>
-      </c>
-      <c r="AH1" s="9">
-        <v>2049</v>
-      </c>
-      <c r="AI1">
-        <v>2050</v>
-      </c>
-    </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,B$1)</f>
-        <v>8.3633611707228332E-6</v>
-      </c>
-      <c r="C2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,C$1)</f>
-        <v>8.1175753380646016E-6</v>
-      </c>
-      <c r="D2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,D$1)</f>
-        <v>7.8717895054063701E-6</v>
-      </c>
-      <c r="E2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,E$1)</f>
-        <v>7.6260036727481386E-6</v>
-      </c>
-      <c r="F2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,F$1)</f>
-        <v>7.3802178400897986E-6</v>
-      </c>
-      <c r="G2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,G$1)</f>
-        <v>7.1344320074315671E-6</v>
-      </c>
-      <c r="H2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,H$1)</f>
-        <v>6.8886461747733356E-6</v>
-      </c>
-      <c r="I2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,I$1)</f>
-        <v>6.642860342115104E-6</v>
-      </c>
-      <c r="J2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,J$1)</f>
-        <v>6.3970745094567641E-6</v>
-      </c>
-      <c r="K2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,K$1)</f>
-        <v>6.1512886767985326E-6</v>
-      </c>
-      <c r="L2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,L$1)</f>
-        <v>5.905502844140301E-6</v>
-      </c>
-      <c r="M2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,M$1)</f>
-        <v>5.6597170114820695E-6</v>
-      </c>
-      <c r="N2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,N$1)</f>
-        <v>5.413931178823838E-6</v>
-      </c>
-      <c r="O2" s="11">
-        <f>TREND('DoE Data'!$B$80:$C$80,'DoE Data'!$B$22:$C$22,O$1)</f>
-        <v>5.168145346165498E-6</v>
-      </c>
-      <c r="P2" s="13">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,P$1)</f>
-        <v>5.0758095874101333E-6</v>
-      </c>
-      <c r="Q2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,Q$1)</f>
-        <v>4.9834738286547143E-6</v>
-      </c>
-      <c r="R2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,R$1)</f>
-        <v>4.8911380698993224E-6</v>
-      </c>
-      <c r="S2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,S$1)</f>
-        <v>4.7988023111439305E-6</v>
-      </c>
-      <c r="T2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,T$1)</f>
-        <v>4.7064665523885386E-6</v>
-      </c>
-      <c r="U2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,U$1)</f>
-        <v>4.6141307936331196E-6</v>
-      </c>
-      <c r="V2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,V$1)</f>
-        <v>4.5217950348777278E-6</v>
-      </c>
-      <c r="W2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,W$1)</f>
-        <v>4.4294592761223359E-6</v>
-      </c>
-      <c r="X2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,X$1)</f>
-        <v>4.3371235173669169E-6</v>
-      </c>
-      <c r="Y2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,Y$1)</f>
-        <v>4.244787758611525E-6</v>
-      </c>
-      <c r="Z2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,Z$1)</f>
-        <v>4.1524519998561331E-6</v>
-      </c>
-      <c r="AA2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,AA$1)</f>
-        <v>4.0601162411007413E-6</v>
-      </c>
-      <c r="AB2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,AB$1)</f>
-        <v>3.9677804823453223E-6</v>
-      </c>
-      <c r="AC2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,AC$1)</f>
-        <v>3.8754447235899304E-6</v>
-      </c>
-      <c r="AD2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,AD$1)</f>
-        <v>3.7831089648345385E-6</v>
-      </c>
-      <c r="AE2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,AE$1)</f>
-        <v>3.6907732060791466E-6</v>
-      </c>
-      <c r="AF2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,AF$1)</f>
-        <v>3.5984374473237277E-6</v>
-      </c>
-      <c r="AG2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,AG$1)</f>
-        <v>3.5061016885683358E-6</v>
-      </c>
-      <c r="AH2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,AH$1)</f>
-        <v>3.4137659298129439E-6</v>
-      </c>
-      <c r="AI2" s="11">
-        <f>TREND('DoE Data'!$C$80:$D$80,'DoE Data'!$C$22:$D$22,AI$1)</f>
-        <v>3.3214301710575249E-6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="C3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="D3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="E3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="F3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="G3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="H3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="I3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="J3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="K3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="L3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="M3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="N3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="O3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="P3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="Q3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="R3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="S3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="T3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="U3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="V3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="W3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="X3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="Y3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="Z3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AA3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AB3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AC3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AD3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AE3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AF3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AG3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AH3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AI3" s="11">
-        <f>'Reformer data'!$B$36</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="11">
-        <f>B3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="C4" s="11">
-        <f>C3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="D4" s="11">
-        <f>D3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="E4" s="11">
-        <f>E3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="F4" s="11">
-        <f>F3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="G4" s="11">
-        <f>G3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="H4" s="11">
-        <f>H3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="I4" s="11">
-        <f>I3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="J4" s="11">
-        <f>J3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="K4" s="11">
-        <f>K3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="L4" s="11">
-        <f>L3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="M4" s="11">
-        <f>M3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="N4" s="11">
-        <f>N3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="O4" s="11">
-        <f>O3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="P4" s="11">
-        <f>P3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="Q4" s="11">
-        <f>Q3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="R4" s="11">
-        <f>R3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="S4" s="11">
-        <f>S3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="T4" s="11">
-        <f>T3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="U4" s="11">
-        <f>U3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="V4" s="11">
-        <f>V3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="W4" s="11">
-        <f>W3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="X4" s="11">
-        <f>X3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="Y4" s="11">
-        <f>Y3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="Z4" s="11">
-        <f>Z3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AA4" s="11">
-        <f>AA3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AB4" s="11">
-        <f>AB3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AC4" s="11">
-        <f>AC3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AD4" s="11">
-        <f>AD3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AE4" s="11">
-        <f>AE3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AF4" s="11">
-        <f>AF3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AG4" s="11">
-        <f>AG3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AH4" s="11">
-        <f>AH3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AI4" s="11">
-        <f>AI3*'IEA Data'!$D$10/'IEA Data'!$D$6</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="11">
-        <f>B4</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="C5" s="11">
-        <f t="shared" ref="C5:AI5" si="0">C4</f>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="D5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="E5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="F5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="G5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="H5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="I5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="J5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="K5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="L5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="M5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="N5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="O5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="P5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="Q5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="R5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="S5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="T5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="U5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="V5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="W5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="X5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="Y5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="Z5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AA5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AB5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AC5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AD5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AE5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AF5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AG5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AH5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-      <c r="AI5" s="11">
-        <f t="shared" si="0"/>
-        <v>4.021408082029495E-6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="11">
-        <f>B3*0.85</f>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="C6">
-        <f t="shared" ref="C6:AI6" si="1">$B6</f>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="D6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="E6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="F6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="G6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="H6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="I6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="J6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="K6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="L6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="M6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="N6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="O6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="P6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="Q6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="R6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="S6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="T6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="U6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="V6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="W6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="X6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="Y6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="Z6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="AA6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="AB6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="AC6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="AD6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="AE6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="AF6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="AG6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="AH6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-      <c r="AI6">
-        <f t="shared" si="1"/>
-        <v>1.1650034275092937E-6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B7" s="11">
-        <f>B2</f>
-        <v>8.3633611707228332E-6</v>
-      </c>
-      <c r="C7" s="11">
-        <f t="shared" ref="C7:AI8" si="2">C2</f>
-        <v>8.1175753380646016E-6</v>
-      </c>
-      <c r="D7" s="11">
-        <f t="shared" si="2"/>
-        <v>7.8717895054063701E-6</v>
-      </c>
-      <c r="E7" s="11">
-        <f t="shared" si="2"/>
-        <v>7.6260036727481386E-6</v>
-      </c>
-      <c r="F7" s="11">
-        <f t="shared" si="2"/>
-        <v>7.3802178400897986E-6</v>
-      </c>
-      <c r="G7" s="11">
-        <f t="shared" si="2"/>
-        <v>7.1344320074315671E-6</v>
-      </c>
-      <c r="H7" s="11">
-        <f t="shared" si="2"/>
-        <v>6.8886461747733356E-6</v>
-      </c>
-      <c r="I7" s="11">
-        <f t="shared" si="2"/>
-        <v>6.642860342115104E-6</v>
-      </c>
-      <c r="J7" s="11">
-        <f t="shared" si="2"/>
-        <v>6.3970745094567641E-6</v>
-      </c>
-      <c r="K7" s="11">
-        <f t="shared" si="2"/>
-        <v>6.1512886767985326E-6</v>
-      </c>
-      <c r="L7" s="11">
-        <f t="shared" si="2"/>
-        <v>5.905502844140301E-6</v>
-      </c>
-      <c r="M7" s="11">
-        <f t="shared" si="2"/>
-        <v>5.6597170114820695E-6</v>
-      </c>
-      <c r="N7" s="11">
-        <f t="shared" si="2"/>
-        <v>5.413931178823838E-6</v>
-      </c>
-      <c r="O7" s="11">
-        <f t="shared" si="2"/>
-        <v>5.168145346165498E-6</v>
-      </c>
-      <c r="P7" s="11">
-        <f t="shared" si="2"/>
-        <v>5.0758095874101333E-6</v>
-      </c>
-      <c r="Q7" s="11">
-        <f t="shared" si="2"/>
-        <v>4.9834738286547143E-6</v>
-      </c>
-      <c r="R7" s="11">
-        <f t="shared" si="2"/>
-        <v>4.8911380698993224E-6</v>
-      </c>
-      <c r="S7" s="11">
-        <f t="shared" si="2"/>
-        <v>4.7988023111439305E-6</v>
-      </c>
-      <c r="T7" s="11">
-        <f t="shared" si="2"/>
-        <v>4.7064665523885386E-6</v>
-      </c>
-      <c r="U7" s="11">
-        <f t="shared" si="2"/>
-        <v>4.6141307936331196E-6</v>
-      </c>
-      <c r="V7" s="11">
-        <f t="shared" si="2"/>
-        <v>4.5217950348777278E-6</v>
-      </c>
-      <c r="W7" s="11">
-        <f t="shared" si="2"/>
-        <v>4.4294592761223359E-6</v>
-      </c>
-      <c r="X7" s="11">
-        <f t="shared" si="2"/>
-        <v>4.3371235173669169E-6</v>
-      </c>
-      <c r="Y7" s="11">
-        <f t="shared" si="2"/>
-        <v>4.244787758611525E-6</v>
-      </c>
-      <c r="Z7" s="11">
-        <f t="shared" si="2"/>
-        <v>4.1524519998561331E-6</v>
-      </c>
-      <c r="AA7" s="11">
-        <f t="shared" si="2"/>
-        <v>4.0601162411007413E-6</v>
-      </c>
-      <c r="AB7" s="11">
-        <f t="shared" si="2"/>
-        <v>3.9677804823453223E-6</v>
-      </c>
-      <c r="AC7" s="11">
-        <f t="shared" si="2"/>
-        <v>3.8754447235899304E-6</v>
-      </c>
-      <c r="AD7" s="11">
-        <f t="shared" si="2"/>
-        <v>3.7831089648345385E-6</v>
-      </c>
-      <c r="AE7" s="11">
-        <f t="shared" si="2"/>
-        <v>3.6907732060791466E-6</v>
-      </c>
-      <c r="AF7" s="11">
-        <f t="shared" si="2"/>
-        <v>3.5984374473237277E-6</v>
-      </c>
-      <c r="AG7" s="11">
-        <f t="shared" si="2"/>
-        <v>3.5061016885683358E-6</v>
-      </c>
-      <c r="AH7" s="11">
-        <f t="shared" si="2"/>
-        <v>3.4137659298129439E-6</v>
-      </c>
-      <c r="AI7" s="11">
-        <f t="shared" si="2"/>
-        <v>3.3214301710575249E-6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B8" s="11">
-        <f>B3</f>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="C8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="D8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="E8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="F8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="G8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="H8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="I8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="J8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="K8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="L8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="M8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="N8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="O8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="P8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="Q8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="R8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="S8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="T8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="U8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="V8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="W8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="X8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="Y8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="Z8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AA8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AB8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AC8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AD8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AE8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AF8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AG8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AH8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
-      <c r="AI8" s="11">
-        <f t="shared" si="2"/>
-        <v>1.3705922676579926E-6</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>